<commit_message>
Document Logistik live, transport T76K912650 and the open P76 steps
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -603,7 +603,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D4" s="6" t="n">
         <v>7</v>
@@ -637,7 +637,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 44 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 16 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 18.</t>
+          <t>Hinter dieser Seite stehen 45 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 16 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 18.</t>
         </is>
       </c>
     </row>
@@ -972,83 +972,83 @@
     <row r="29" ht="20" customHeight="1">
       <c r="B29" s="16" t="inlineStr">
         <is>
+          <t>Logistik live: Kommissionierung und Produktion fast in Echtzeit</t>
+        </is>
+      </c>
+      <c r="C29" s="20" t="inlineStr">
+        <is>
+          <t>Läuft</t>
+        </is>
+      </c>
+      <c r="D29" s="16" t="inlineStr">
+        <is>
+          <t>Transport nach P76 (Ingo)</t>
+        </is>
+      </c>
+      <c r="E29" s="18" t="inlineStr">
+        <is>
+          <t>01.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="B30" s="16" t="inlineStr">
+        <is>
           <t>Zwei kleine Entscheide (Beschriftung, SAP-Schlüssel)</t>
         </is>
       </c>
-      <c r="C29" s="21" t="inlineStr">
+      <c r="C30" s="21" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="D29" s="16" t="inlineStr">
+      <c r="D30" s="16" t="inlineStr">
         <is>
           <t>Ingo</t>
         </is>
       </c>
-      <c r="E29" s="18" t="inlineStr">
+      <c r="E30" s="18" t="inlineStr">
         <is>
           <t>29.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="B31" s="14" t="inlineStr">
+    <row r="32" ht="22" customHeight="1">
+      <c r="B32" s="14" t="inlineStr">
         <is>
           <t>SAP</t>
         </is>
       </c>
-      <c r="C31" s="15" t="n"/>
-      <c r="D31" s="15" t="n"/>
-      <c r="E31" s="15" t="n"/>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="B32" s="16" t="inlineStr">
-        <is>
-          <t>ZZPRDAT Produktionsdatum: gemeinsamer Test</t>
-        </is>
-      </c>
-      <c r="C32" s="20" t="inlineStr">
-        <is>
-          <t>Läuft</t>
-        </is>
-      </c>
-      <c r="D32" s="16" t="inlineStr">
-        <is>
-          <t>Test 12.10. (Lucas, Marco, Adil)</t>
-        </is>
-      </c>
-      <c r="E32" s="18" t="inlineStr">
-        <is>
-          <t>01.10.2026</t>
-        </is>
-      </c>
+      <c r="C32" s="15" t="n"/>
+      <c r="D32" s="15" t="n"/>
+      <c r="E32" s="15" t="n"/>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="B33" s="16" t="inlineStr">
         <is>
-          <t>ZLO03 Mengen und Materialien: Test und Transport</t>
-        </is>
-      </c>
-      <c r="C33" s="21" t="inlineStr">
-        <is>
-          <t>Offen</t>
+          <t>ZZPRDAT Produktionsdatum: gemeinsamer Test</t>
+        </is>
+      </c>
+      <c r="C33" s="20" t="inlineStr">
+        <is>
+          <t>Läuft</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
         <is>
-          <t>Ingo</t>
+          <t>Test 12.10. (Lucas, Marco, Adil)</t>
         </is>
       </c>
       <c r="E33" s="18" t="inlineStr">
         <is>
-          <t>14.08.2026</t>
+          <t>01.10.2026</t>
         </is>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="B34" s="16" t="inlineStr">
         <is>
-          <t>ZC12 Nullmengen: Fehlersuche einschalten</t>
+          <t>ZLO03 Mengen und Materialien: Test und Transport</t>
         </is>
       </c>
       <c r="C34" s="21" t="inlineStr">
@@ -1063,162 +1063,184 @@
       </c>
       <c r="E34" s="18" t="inlineStr">
         <is>
-          <t>07.09.2026</t>
+          <t>14.08.2026</t>
         </is>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="B35" s="16" t="inlineStr">
         <is>
+          <t>ZC12 Nullmengen: Fehlersuche einschalten</t>
+        </is>
+      </c>
+      <c r="C35" s="21" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="D35" s="16" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="E35" s="18" t="inlineStr">
+        <is>
+          <t>07.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="B36" s="16" t="inlineStr">
+        <is>
           <t>ZRL2 Mengenrabatt Trafag AT</t>
         </is>
       </c>
-      <c r="C35" s="17" t="inlineStr">
+      <c r="C36" s="17" t="inlineStr">
         <is>
           <t>Bereit</t>
         </is>
       </c>
-      <c r="D35" s="16" t="inlineStr"/>
-      <c r="E35" s="18" t="inlineStr">
+      <c r="D36" s="16" t="inlineStr"/>
+      <c r="E36" s="18" t="inlineStr">
         <is>
           <t>30.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="22" customHeight="1">
-      <c r="B37" s="14" t="inlineStr">
+    <row r="38" ht="22" customHeight="1">
+      <c r="B38" s="14" t="inlineStr">
         <is>
           <t>Railway</t>
         </is>
       </c>
-      <c r="C37" s="15" t="n"/>
-      <c r="D37" s="15" t="n"/>
-      <c r="E37" s="15" t="n"/>
-    </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="B38" s="16" t="inlineStr">
-        <is>
-          <t>Umsatz-Gesamtsicht aller Standorte</t>
-        </is>
-      </c>
-      <c r="C38" s="17" t="inlineStr">
-        <is>
-          <t>Bereit</t>
-        </is>
-      </c>
-      <c r="D38" s="16" t="inlineStr"/>
-      <c r="E38" s="18" t="inlineStr">
-        <is>
-          <t>29.09.2026</t>
-        </is>
-      </c>
+      <c r="C38" s="15" t="n"/>
+      <c r="D38" s="15" t="n"/>
+      <c r="E38" s="15" t="n"/>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="B39" s="16" t="inlineStr">
         <is>
+          <t>Umsatz-Gesamtsicht aller Standorte</t>
+        </is>
+      </c>
+      <c r="C39" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D39" s="16" t="inlineStr"/>
+      <c r="E39" s="18" t="inlineStr">
+        <is>
+          <t>29.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="B40" s="16" t="inlineStr">
+        <is>
           <t>Top-15-Kunden und Schweiz bestätigen</t>
         </is>
       </c>
-      <c r="C39" s="19" t="inlineStr">
+      <c r="C40" s="19" t="inlineStr">
         <is>
           <t>Wartet</t>
         </is>
       </c>
-      <c r="D39" s="16" t="inlineStr">
+      <c r="D40" s="16" t="inlineStr">
         <is>
           <t>Andreas / Patrik</t>
         </is>
       </c>
-      <c r="E39" s="18" t="inlineStr">
+      <c r="E40" s="18" t="inlineStr">
         <is>
           <t>29.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="22" customHeight="1">
-      <c r="B41" s="14" t="inlineStr">
+    <row r="42" ht="22" customHeight="1">
+      <c r="B42" s="14" t="inlineStr">
         <is>
           <t>Plattform</t>
         </is>
       </c>
-      <c r="C41" s="15" t="n"/>
-      <c r="D41" s="15" t="n"/>
-      <c r="E41" s="15" t="n"/>
-    </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="B42" s="16" t="inlineStr">
-        <is>
-          <t>Webapp schneller</t>
-        </is>
-      </c>
-      <c r="C42" s="17" t="inlineStr">
-        <is>
-          <t>Bereit</t>
-        </is>
-      </c>
-      <c r="D42" s="16" t="inlineStr"/>
-      <c r="E42" s="18" t="inlineStr">
-        <is>
-          <t>28.09.2026</t>
-        </is>
-      </c>
+      <c r="C42" s="15" t="n"/>
+      <c r="D42" s="15" t="n"/>
+      <c r="E42" s="15" t="n"/>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="B43" s="16" t="inlineStr">
         <is>
+          <t>Webapp schneller</t>
+        </is>
+      </c>
+      <c r="C43" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D43" s="16" t="inlineStr"/>
+      <c r="E43" s="18" t="inlineStr">
+        <is>
+          <t>28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="B44" s="16" t="inlineStr">
+        <is>
           <t>Server im Dauerbetrieb</t>
         </is>
       </c>
-      <c r="C43" s="19" t="inlineStr">
+      <c r="C44" s="19" t="inlineStr">
         <is>
           <t>Wartet</t>
         </is>
       </c>
-      <c r="D43" s="16" t="inlineStr">
+      <c r="D44" s="16" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="E43" s="18" t="inlineStr">
+      <c r="E44" s="18" t="inlineStr">
         <is>
           <t>28.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="22" customHeight="1">
-      <c r="B45" s="14" t="inlineStr">
+    <row r="46" ht="22" customHeight="1">
+      <c r="B46" s="14" t="inlineStr">
         <is>
           <t>Projekte</t>
         </is>
       </c>
-      <c r="C45" s="15" t="n"/>
-      <c r="D45" s="15" t="n"/>
-      <c r="E45" s="15" t="n"/>
-    </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="B46" s="16" t="inlineStr">
+      <c r="C46" s="15" t="n"/>
+      <c r="D46" s="15" t="n"/>
+      <c r="E46" s="15" t="n"/>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="B47" s="16" t="inlineStr">
         <is>
           <t>Smartsheet-Ablösung, Power-BI-Verantwortliche, Data Lake</t>
         </is>
       </c>
-      <c r="C46" s="21" t="inlineStr">
+      <c r="C47" s="21" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="D46" s="16" t="inlineStr">
+      <c r="D47" s="16" t="inlineStr">
         <is>
           <t>noch nicht gestartet</t>
         </is>
       </c>
-      <c r="E46" s="18" t="inlineStr">
+      <c r="E47" s="18" t="inlineStr">
         <is>
           <t>29.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="26" customHeight="1">
-      <c r="B48" s="22" t="inlineStr">
+    <row r="49" ht="26" customHeight="1">
+      <c r="B49" s="22" t="inlineStr">
         <is>
           <t>Bereit = erledigt und in Betrieb · Läuft = in Arbeit · Wartet = braucht eine andere Person · Offen = noch nicht begonnen oder Entscheid von Ingo. Details und Nachweise: Wochen_Todo.xlsx.</t>
         </is>
@@ -1227,7 +1249,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B48:E48"/>
+    <mergeCell ref="B49:E49"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Record Logistik live in P76 and the 15:01 deploy
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -600,10 +600,10 @@
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="B4" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D4" s="6" t="n">
         <v>7</v>
@@ -975,16 +975,12 @@
           <t>Logistik live: Kommissionierung und Produktion fast in Echtzeit</t>
         </is>
       </c>
-      <c r="C29" s="20" t="inlineStr">
-        <is>
-          <t>Läuft</t>
-        </is>
-      </c>
-      <c r="D29" s="16" t="inlineStr">
-        <is>
-          <t>Transport nach P76 (Ingo)</t>
-        </is>
-      </c>
+      <c r="C29" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D29" s="16" t="inlineStr"/>
       <c r="E29" s="18" t="inlineStr">
         <is>
           <t>01.10.2026</t>

</xml_diff>

<commit_message>
Document Verwendung & Risiko, the data limits behind it and the 16:05 deploy
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -600,7 +600,7 @@
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="B4" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" s="5" t="n">
         <v>2</v>
@@ -637,7 +637,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 45 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 16 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 18.</t>
+          <t>Hinter dieser Seite stehen 45 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 16 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 19.</t>
         </is>
       </c>
     </row>
@@ -990,83 +990,79 @@
     <row r="30" ht="20" customHeight="1">
       <c r="B30" s="16" t="inlineStr">
         <is>
+          <t>Stückliste: Verwendung &amp; Risiko über mehrere Stufen</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D30" s="16" t="inlineStr"/>
+      <c r="E30" s="18" t="inlineStr">
+        <is>
+          <t>01.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="B31" s="16" t="inlineStr">
+        <is>
           <t>Zwei kleine Entscheide (Beschriftung, SAP-Schlüssel)</t>
         </is>
       </c>
-      <c r="C30" s="21" t="inlineStr">
+      <c r="C31" s="21" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="D30" s="16" t="inlineStr">
+      <c r="D31" s="16" t="inlineStr">
         <is>
           <t>Ingo</t>
         </is>
       </c>
-      <c r="E30" s="18" t="inlineStr">
+      <c r="E31" s="18" t="inlineStr">
         <is>
           <t>29.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="B32" s="14" t="inlineStr">
+    <row r="33" ht="22" customHeight="1">
+      <c r="B33" s="14" t="inlineStr">
         <is>
           <t>SAP</t>
         </is>
       </c>
-      <c r="C32" s="15" t="n"/>
-      <c r="D32" s="15" t="n"/>
-      <c r="E32" s="15" t="n"/>
-    </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="B33" s="16" t="inlineStr">
-        <is>
-          <t>ZZPRDAT Produktionsdatum: gemeinsamer Test</t>
-        </is>
-      </c>
-      <c r="C33" s="20" t="inlineStr">
-        <is>
-          <t>Läuft</t>
-        </is>
-      </c>
-      <c r="D33" s="16" t="inlineStr">
-        <is>
-          <t>Test 12.10. (Lucas, Marco, Adil)</t>
-        </is>
-      </c>
-      <c r="E33" s="18" t="inlineStr">
-        <is>
-          <t>01.10.2026</t>
-        </is>
-      </c>
+      <c r="C33" s="15" t="n"/>
+      <c r="D33" s="15" t="n"/>
+      <c r="E33" s="15" t="n"/>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="B34" s="16" t="inlineStr">
         <is>
-          <t>ZLO03 Mengen und Materialien: Test und Transport</t>
-        </is>
-      </c>
-      <c r="C34" s="21" t="inlineStr">
-        <is>
-          <t>Offen</t>
+          <t>ZZPRDAT Produktionsdatum: gemeinsamer Test</t>
+        </is>
+      </c>
+      <c r="C34" s="20" t="inlineStr">
+        <is>
+          <t>Läuft</t>
         </is>
       </c>
       <c r="D34" s="16" t="inlineStr">
         <is>
-          <t>Ingo</t>
+          <t>Test 12.10. (Lucas, Marco, Adil)</t>
         </is>
       </c>
       <c r="E34" s="18" t="inlineStr">
         <is>
-          <t>14.08.2026</t>
+          <t>01.10.2026</t>
         </is>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="B35" s="16" t="inlineStr">
         <is>
-          <t>ZC12 Nullmengen: Fehlersuche einschalten</t>
+          <t>ZLO03 Mengen und Materialien: Test und Transport</t>
         </is>
       </c>
       <c r="C35" s="21" t="inlineStr">
@@ -1081,162 +1077,184 @@
       </c>
       <c r="E35" s="18" t="inlineStr">
         <is>
-          <t>07.09.2026</t>
+          <t>14.08.2026</t>
         </is>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="B36" s="16" t="inlineStr">
         <is>
+          <t>ZC12 Nullmengen: Fehlersuche einschalten</t>
+        </is>
+      </c>
+      <c r="C36" s="21" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="D36" s="16" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="E36" s="18" t="inlineStr">
+        <is>
+          <t>07.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="B37" s="16" t="inlineStr">
+        <is>
           <t>ZRL2 Mengenrabatt Trafag AT</t>
         </is>
       </c>
-      <c r="C36" s="17" t="inlineStr">
+      <c r="C37" s="17" t="inlineStr">
         <is>
           <t>Bereit</t>
         </is>
       </c>
-      <c r="D36" s="16" t="inlineStr"/>
-      <c r="E36" s="18" t="inlineStr">
+      <c r="D37" s="16" t="inlineStr"/>
+      <c r="E37" s="18" t="inlineStr">
         <is>
           <t>30.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="22" customHeight="1">
-      <c r="B38" s="14" t="inlineStr">
+    <row r="39" ht="22" customHeight="1">
+      <c r="B39" s="14" t="inlineStr">
         <is>
           <t>Railway</t>
         </is>
       </c>
-      <c r="C38" s="15" t="n"/>
-      <c r="D38" s="15" t="n"/>
-      <c r="E38" s="15" t="n"/>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="B39" s="16" t="inlineStr">
-        <is>
-          <t>Umsatz-Gesamtsicht aller Standorte</t>
-        </is>
-      </c>
-      <c r="C39" s="17" t="inlineStr">
-        <is>
-          <t>Bereit</t>
-        </is>
-      </c>
-      <c r="D39" s="16" t="inlineStr"/>
-      <c r="E39" s="18" t="inlineStr">
-        <is>
-          <t>29.09.2026</t>
-        </is>
-      </c>
+      <c r="C39" s="15" t="n"/>
+      <c r="D39" s="15" t="n"/>
+      <c r="E39" s="15" t="n"/>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="B40" s="16" t="inlineStr">
         <is>
+          <t>Umsatz-Gesamtsicht aller Standorte</t>
+        </is>
+      </c>
+      <c r="C40" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D40" s="16" t="inlineStr"/>
+      <c r="E40" s="18" t="inlineStr">
+        <is>
+          <t>29.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="B41" s="16" t="inlineStr">
+        <is>
           <t>Top-15-Kunden und Schweiz bestätigen</t>
         </is>
       </c>
-      <c r="C40" s="19" t="inlineStr">
+      <c r="C41" s="19" t="inlineStr">
         <is>
           <t>Wartet</t>
         </is>
       </c>
-      <c r="D40" s="16" t="inlineStr">
+      <c r="D41" s="16" t="inlineStr">
         <is>
           <t>Andreas / Patrik</t>
         </is>
       </c>
-      <c r="E40" s="18" t="inlineStr">
+      <c r="E41" s="18" t="inlineStr">
         <is>
           <t>29.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="22" customHeight="1">
-      <c r="B42" s="14" t="inlineStr">
+    <row r="43" ht="22" customHeight="1">
+      <c r="B43" s="14" t="inlineStr">
         <is>
           <t>Plattform</t>
         </is>
       </c>
-      <c r="C42" s="15" t="n"/>
-      <c r="D42" s="15" t="n"/>
-      <c r="E42" s="15" t="n"/>
-    </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="B43" s="16" t="inlineStr">
-        <is>
-          <t>Webapp schneller</t>
-        </is>
-      </c>
-      <c r="C43" s="17" t="inlineStr">
-        <is>
-          <t>Bereit</t>
-        </is>
-      </c>
-      <c r="D43" s="16" t="inlineStr"/>
-      <c r="E43" s="18" t="inlineStr">
-        <is>
-          <t>28.09.2026</t>
-        </is>
-      </c>
+      <c r="C43" s="15" t="n"/>
+      <c r="D43" s="15" t="n"/>
+      <c r="E43" s="15" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="B44" s="16" t="inlineStr">
         <is>
+          <t>Webapp schneller</t>
+        </is>
+      </c>
+      <c r="C44" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D44" s="16" t="inlineStr"/>
+      <c r="E44" s="18" t="inlineStr">
+        <is>
+          <t>28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="B45" s="16" t="inlineStr">
+        <is>
           <t>Server im Dauerbetrieb</t>
         </is>
       </c>
-      <c r="C44" s="19" t="inlineStr">
+      <c r="C45" s="19" t="inlineStr">
         <is>
           <t>Wartet</t>
         </is>
       </c>
-      <c r="D44" s="16" t="inlineStr">
+      <c r="D45" s="16" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="E44" s="18" t="inlineStr">
+      <c r="E45" s="18" t="inlineStr">
         <is>
           <t>28.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="22" customHeight="1">
-      <c r="B46" s="14" t="inlineStr">
+    <row r="47" ht="22" customHeight="1">
+      <c r="B47" s="14" t="inlineStr">
         <is>
           <t>Projekte</t>
         </is>
       </c>
-      <c r="C46" s="15" t="n"/>
-      <c r="D46" s="15" t="n"/>
-      <c r="E46" s="15" t="n"/>
-    </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="B47" s="16" t="inlineStr">
+      <c r="C47" s="15" t="n"/>
+      <c r="D47" s="15" t="n"/>
+      <c r="E47" s="15" t="n"/>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="B48" s="16" t="inlineStr">
         <is>
           <t>Smartsheet-Ablösung, Power-BI-Verantwortliche, Data Lake</t>
         </is>
       </c>
-      <c r="C47" s="21" t="inlineStr">
+      <c r="C48" s="21" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="D47" s="16" t="inlineStr">
+      <c r="D48" s="16" t="inlineStr">
         <is>
           <t>noch nicht gestartet</t>
         </is>
       </c>
-      <c r="E47" s="18" t="inlineStr">
+      <c r="E48" s="18" t="inlineStr">
         <is>
           <t>29.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="26" customHeight="1">
-      <c r="B49" s="22" t="inlineStr">
+    <row r="50" ht="26" customHeight="1">
+      <c r="B50" s="22" t="inlineStr">
         <is>
           <t>Bereit = erledigt und in Betrieb · Läuft = in Arbeit · Wartet = braucht eine andere Person · Offen = noch nicht begonnen oder Entscheid von Ingo. Details und Nachweise: Wochen_Todo.xlsx.</t>
         </is>
@@ -1245,7 +1263,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B49:E49"/>
+    <mergeCell ref="B50:E50"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Document the Netzwerk tab, its probe rules and the 07:20 deploy
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -591,7 +591,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Stand 01.10.2026  ·  Ingo Kohler</t>
+          <t>Stand 02.10.2026  ·  Ingo Kohler</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -600,13 +600,13 @@
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="B4" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C4" s="5" t="n">
         <v>2</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E4" s="7" t="n">
         <v>4</v>
@@ -637,7 +637,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 45 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 16 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 19.</t>
+          <t>Hinter dieser Seite stehen 46 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 16 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 19.</t>
         </is>
       </c>
     </row>
@@ -1202,59 +1202,99 @@
     <row r="45" ht="20" customHeight="1">
       <c r="B45" s="16" t="inlineStr">
         <is>
+          <t>Netzwerk-Reiter: Netzkarte, Verfügbarkeit, Netz oder Daten, Sicherheit</t>
+        </is>
+      </c>
+      <c r="C45" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D45" s="16" t="inlineStr"/>
+      <c r="E45" s="18" t="inlineStr">
+        <is>
+          <t>02.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="B46" s="16" t="inlineStr">
+        <is>
+          <t>AD-Computerkonten im Netzwerk-Reiter einschalten</t>
+        </is>
+      </c>
+      <c r="C46" s="19" t="inlineStr">
+        <is>
+          <t>Wartet</t>
+        </is>
+      </c>
+      <c r="D46" s="16" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="E46" s="18" t="inlineStr">
+        <is>
+          <t>02.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="B47" s="16" t="inlineStr">
+        <is>
           <t>Server im Dauerbetrieb</t>
         </is>
       </c>
-      <c r="C45" s="19" t="inlineStr">
+      <c r="C47" s="19" t="inlineStr">
         <is>
           <t>Wartet</t>
         </is>
       </c>
-      <c r="D45" s="16" t="inlineStr">
+      <c r="D47" s="16" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="E45" s="18" t="inlineStr">
+      <c r="E47" s="18" t="inlineStr">
         <is>
           <t>28.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="22" customHeight="1">
-      <c r="B47" s="14" t="inlineStr">
+    <row r="49" ht="22" customHeight="1">
+      <c r="B49" s="14" t="inlineStr">
         <is>
           <t>Projekte</t>
         </is>
       </c>
-      <c r="C47" s="15" t="n"/>
-      <c r="D47" s="15" t="n"/>
-      <c r="E47" s="15" t="n"/>
-    </row>
-    <row r="48" ht="20" customHeight="1">
-      <c r="B48" s="16" t="inlineStr">
+      <c r="C49" s="15" t="n"/>
+      <c r="D49" s="15" t="n"/>
+      <c r="E49" s="15" t="n"/>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="B50" s="16" t="inlineStr">
         <is>
           <t>Smartsheet-Ablösung, Power-BI-Verantwortliche, Data Lake</t>
         </is>
       </c>
-      <c r="C48" s="21" t="inlineStr">
+      <c r="C50" s="21" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="D48" s="16" t="inlineStr">
+      <c r="D50" s="16" t="inlineStr">
         <is>
           <t>noch nicht gestartet</t>
         </is>
       </c>
-      <c r="E48" s="18" t="inlineStr">
+      <c r="E50" s="18" t="inlineStr">
         <is>
           <t>29.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="26" customHeight="1">
-      <c r="B50" s="22" t="inlineStr">
+    <row r="52" ht="26" customHeight="1">
+      <c r="B52" s="22" t="inlineStr">
         <is>
           <t>Bereit = erledigt und in Betrieb · Läuft = in Arbeit · Wartet = braucht eine andere Person · Offen = noch nicht begonnen oder Entscheid von Ingo. Details und Nachweise: Wochen_Todo.xlsx.</t>
         </is>
@@ -1263,7 +1303,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B50:E50"/>
+    <mergeCell ref="B52:E52"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Document the AD switch in the Netzwerk tab and the 07:34 deploy
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -139,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -196,6 +196,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -606,7 +609,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E4" s="7" t="n">
         <v>4</v>
@@ -1223,16 +1226,12 @@
           <t>AD-Computerkonten im Netzwerk-Reiter einschalten</t>
         </is>
       </c>
-      <c r="C46" s="19" t="inlineStr">
-        <is>
-          <t>Wartet</t>
-        </is>
-      </c>
-      <c r="D46" s="16" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
+      <c r="C46" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D46" s="16" t="inlineStr"/>
       <c r="E46" s="18" t="inlineStr">
         <is>
           <t>02.10.2026</t>
@@ -1294,7 +1293,7 @@
       </c>
     </row>
     <row r="52" ht="26" customHeight="1">
-      <c r="B52" s="22" t="inlineStr">
+      <c r="B52" s="23" t="inlineStr">
         <is>
           <t>Bereit = erledigt und in Betrieb · Läuft = in Arbeit · Wartet = braucht eine andere Person · Offen = noch nicht begonnen oder Entscheid von Ingo. Details und Nachweise: Wochen_Todo.xlsx.</t>
         </is>

</xml_diff>

<commit_message>
Document the Verkauf tab and the 13:24 deploy
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -569,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -603,7 +603,7 @@
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="B4" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C4" s="5" t="n">
         <v>2</v>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 46 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 16 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 19.</t>
+          <t>Hinter dieser Seite stehen 47 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 16 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 19.</t>
         </is>
       </c>
     </row>
@@ -785,7 +785,7 @@
     <row r="17" ht="22" customHeight="1">
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Verkauf</t>
         </is>
       </c>
       <c r="C17" s="15" t="n"/>
@@ -795,7 +795,7 @@
     <row r="18" ht="20" customHeight="1">
       <c r="B18" s="16" t="inlineStr">
         <is>
-          <t>Kader 8,1 h, übrige 8,0 h je Arbeitstag</t>
+          <t>Reiter Verkauf: Kunden, Rückgang, Konzentration, Cross-Selling, Preise, Prognose, Weltkarte</t>
         </is>
       </c>
       <c r="C18" s="17" t="inlineStr">
@@ -803,53 +803,31 @@
           <t>Bereit</t>
         </is>
       </c>
-      <c r="D18" s="16" t="inlineStr"/>
+      <c r="D18" s="16" t="inlineStr">
+        <is>
+          <t>Sichtprüfung Ingo</t>
+        </is>
+      </c>
       <c r="E18" s="18" t="inlineStr">
         <is>
-          <t>01.10.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="B19" s="16" t="inlineStr">
-        <is>
-          <t>Abwesenheiten mit Von/Bis, nur genehmigte, Krankenquote je Zeitraum</t>
-        </is>
-      </c>
-      <c r="C19" s="17" t="inlineStr">
-        <is>
-          <t>Bereit</t>
-        </is>
-      </c>
-      <c r="D19" s="16" t="inlineStr"/>
-      <c r="E19" s="18" t="inlineStr">
-        <is>
-          <t>01.10.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="B20" s="16" t="inlineStr">
-        <is>
-          <t>Absenz-Ampel: bis 4,99 % gelb, ab 5 % rot</t>
-        </is>
-      </c>
-      <c r="C20" s="17" t="inlineStr">
-        <is>
-          <t>Bereit</t>
-        </is>
-      </c>
-      <c r="D20" s="16" t="inlineStr"/>
-      <c r="E20" s="18" t="inlineStr">
-        <is>
-          <t>01.10.2026</t>
-        </is>
-      </c>
+          <t>02.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="n"/>
+      <c r="D20" s="15" t="n"/>
+      <c r="E20" s="15" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="B21" s="16" t="inlineStr">
         <is>
-          <t>SAP-Daten täglich automatisch</t>
+          <t>Kader 8,1 h, übrige 8,0 h je Arbeitstag</t>
         </is>
       </c>
       <c r="C21" s="17" t="inlineStr">
@@ -867,115 +845,115 @@
     <row r="22" ht="20" customHeight="1">
       <c r="B22" s="16" t="inlineStr">
         <is>
-          <t>Rexx-Berichte täglich automatisch</t>
-        </is>
-      </c>
-      <c r="C22" s="19" t="inlineStr">
-        <is>
-          <t>Wartet</t>
-        </is>
-      </c>
-      <c r="D22" s="16" t="inlineStr">
-        <is>
-          <t>Upgreat</t>
-        </is>
-      </c>
+          <t>Abwesenheiten mit Von/Bis, nur genehmigte, Krankenquote je Zeitraum</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D22" s="16" t="inlineStr"/>
       <c r="E22" s="18" t="inlineStr">
         <is>
-          <t>30.09.2026</t>
+          <t>01.10.2026</t>
         </is>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="B23" s="16" t="inlineStr">
         <is>
-          <t>Krankheitsarten bestätigen</t>
-        </is>
-      </c>
-      <c r="C23" s="19" t="inlineStr">
+          <t>Absenz-Ampel: bis 4,99 % gelb, ab 5 % rot</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr"/>
+      <c r="E23" s="18" t="inlineStr">
+        <is>
+          <t>01.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>SAP-Daten täglich automatisch</t>
+        </is>
+      </c>
+      <c r="C24" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr"/>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>01.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>Rexx-Berichte täglich automatisch</t>
+        </is>
+      </c>
+      <c r="C25" s="19" t="inlineStr">
         <is>
           <t>Wartet</t>
         </is>
       </c>
-      <c r="D23" s="16" t="inlineStr">
-        <is>
-          <t>Sonja</t>
-        </is>
-      </c>
-      <c r="E23" s="18" t="inlineStr">
-        <is>
-          <t>01.10.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="B25" s="14" t="inlineStr">
-        <is>
-          <t>Einkauf</t>
-        </is>
-      </c>
-      <c r="C25" s="15" t="n"/>
-      <c r="D25" s="15" t="n"/>
-      <c r="E25" s="15" t="n"/>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>Upgreat</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>30.09.2026</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="B26" s="16" t="inlineStr">
         <is>
-          <t>Seite nach dem Auffrischen sofort da</t>
-        </is>
-      </c>
-      <c r="C26" s="17" t="inlineStr">
-        <is>
-          <t>Bereit</t>
-        </is>
-      </c>
-      <c r="D26" s="16" t="inlineStr"/>
+          <t>Krankheitsarten bestätigen</t>
+        </is>
+      </c>
+      <c r="C26" s="19" t="inlineStr">
+        <is>
+          <t>Wartet</t>
+        </is>
+      </c>
+      <c r="D26" s="16" t="inlineStr">
+        <is>
+          <t>Sonja</t>
+        </is>
+      </c>
       <c r="E26" s="18" t="inlineStr">
         <is>
           <t>01.10.2026</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="B27" s="16" t="inlineStr">
-        <is>
-          <t>Lagerwert-Verlauf je Woche</t>
-        </is>
-      </c>
-      <c r="C27" s="17" t="inlineStr">
-        <is>
-          <t>Bereit</t>
-        </is>
-      </c>
-      <c r="D27" s="16" t="inlineStr"/>
-      <c r="E27" s="18" t="inlineStr">
-        <is>
-          <t>28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="B28" s="16" t="inlineStr">
-        <is>
-          <t>Texte Produktgruppen D1/D5</t>
-        </is>
-      </c>
-      <c r="C28" s="17" t="inlineStr">
-        <is>
-          <t>Bereit</t>
-        </is>
-      </c>
-      <c r="D28" s="16" t="inlineStr"/>
-      <c r="E28" s="18" t="inlineStr">
-        <is>
-          <t>01.10.2026</t>
-        </is>
-      </c>
+    <row r="28" ht="22" customHeight="1">
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>Einkauf</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="n"/>
+      <c r="D28" s="15" t="n"/>
+      <c r="E28" s="15" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="B29" s="16" t="inlineStr">
         <is>
-          <t>Logistik live: Kommissionierung und Produktion fast in Echtzeit</t>
+          <t>Seite nach dem Auffrischen sofort da</t>
         </is>
       </c>
       <c r="C29" s="17" t="inlineStr">
@@ -993,7 +971,7 @@
     <row r="30" ht="20" customHeight="1">
       <c r="B30" s="16" t="inlineStr">
         <is>
-          <t>Stückliste: Verwendung &amp; Risiko über mehrere Stufen</t>
+          <t>Lagerwert-Verlauf je Woche</t>
         </is>
       </c>
       <c r="C30" s="17" t="inlineStr">
@@ -1004,140 +982,166 @@
       <c r="D30" s="16" t="inlineStr"/>
       <c r="E30" s="18" t="inlineStr">
         <is>
-          <t>01.10.2026</t>
+          <t>28.09.2026</t>
         </is>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="B31" s="16" t="inlineStr">
         <is>
-          <t>Zwei kleine Entscheide (Beschriftung, SAP-Schlüssel)</t>
-        </is>
-      </c>
-      <c r="C31" s="21" t="inlineStr">
-        <is>
-          <t>Offen</t>
-        </is>
-      </c>
-      <c r="D31" s="16" t="inlineStr">
-        <is>
-          <t>Ingo</t>
-        </is>
-      </c>
+          <t>Texte Produktgruppen D1/D5</t>
+        </is>
+      </c>
+      <c r="C31" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="18" t="inlineStr">
         <is>
-          <t>29.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="22" customHeight="1">
-      <c r="B33" s="14" t="inlineStr">
-        <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="C33" s="15" t="n"/>
-      <c r="D33" s="15" t="n"/>
-      <c r="E33" s="15" t="n"/>
+          <t>01.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="B32" s="16" t="inlineStr">
+        <is>
+          <t>Logistik live: Kommissionierung und Produktion fast in Echtzeit</t>
+        </is>
+      </c>
+      <c r="C32" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D32" s="16" t="inlineStr"/>
+      <c r="E32" s="18" t="inlineStr">
+        <is>
+          <t>01.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="B33" s="16" t="inlineStr">
+        <is>
+          <t>Stückliste: Verwendung &amp; Risiko über mehrere Stufen</t>
+        </is>
+      </c>
+      <c r="C33" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D33" s="16" t="inlineStr"/>
+      <c r="E33" s="18" t="inlineStr">
+        <is>
+          <t>01.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="B34" s="16" t="inlineStr">
         <is>
-          <t>ZZPRDAT Produktionsdatum: gemeinsamer Test</t>
-        </is>
-      </c>
-      <c r="C34" s="20" t="inlineStr">
-        <is>
-          <t>Läuft</t>
+          <t>Zwei kleine Entscheide (Beschriftung, SAP-Schlüssel)</t>
+        </is>
+      </c>
+      <c r="C34" s="21" t="inlineStr">
+        <is>
+          <t>Offen</t>
         </is>
       </c>
       <c r="D34" s="16" t="inlineStr">
         <is>
-          <t>Test 12.10. (Lucas, Marco, Adil)</t>
+          <t>Ingo</t>
         </is>
       </c>
       <c r="E34" s="18" t="inlineStr">
         <is>
-          <t>01.10.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="B35" s="16" t="inlineStr">
-        <is>
-          <t>ZLO03 Mengen und Materialien: Test und Transport</t>
-        </is>
-      </c>
-      <c r="C35" s="21" t="inlineStr">
-        <is>
-          <t>Offen</t>
-        </is>
-      </c>
-      <c r="D35" s="16" t="inlineStr">
-        <is>
-          <t>Ingo</t>
-        </is>
-      </c>
-      <c r="E35" s="18" t="inlineStr">
-        <is>
-          <t>14.08.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="B36" s="16" t="inlineStr">
-        <is>
-          <t>ZC12 Nullmengen: Fehlersuche einschalten</t>
-        </is>
-      </c>
-      <c r="C36" s="21" t="inlineStr">
-        <is>
-          <t>Offen</t>
-        </is>
-      </c>
-      <c r="D36" s="16" t="inlineStr">
-        <is>
-          <t>Ingo</t>
-        </is>
-      </c>
-      <c r="E36" s="18" t="inlineStr">
-        <is>
-          <t>07.09.2026</t>
-        </is>
-      </c>
+          <t>29.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="C36" s="15" t="n"/>
+      <c r="D36" s="15" t="n"/>
+      <c r="E36" s="15" t="n"/>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="B37" s="16" t="inlineStr">
         <is>
-          <t>ZRL2 Mengenrabatt Trafag AT</t>
-        </is>
-      </c>
-      <c r="C37" s="17" t="inlineStr">
-        <is>
-          <t>Bereit</t>
-        </is>
-      </c>
-      <c r="D37" s="16" t="inlineStr"/>
+          <t>ZZPRDAT Produktionsdatum: gemeinsamer Test</t>
+        </is>
+      </c>
+      <c r="C37" s="20" t="inlineStr">
+        <is>
+          <t>Läuft</t>
+        </is>
+      </c>
+      <c r="D37" s="16" t="inlineStr">
+        <is>
+          <t>Test 12.10. (Lucas, Marco, Adil)</t>
+        </is>
+      </c>
       <c r="E37" s="18" t="inlineStr">
         <is>
-          <t>30.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="22" customHeight="1">
-      <c r="B39" s="14" t="inlineStr">
-        <is>
-          <t>Railway</t>
-        </is>
-      </c>
-      <c r="C39" s="15" t="n"/>
-      <c r="D39" s="15" t="n"/>
-      <c r="E39" s="15" t="n"/>
+          <t>01.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="B38" s="16" t="inlineStr">
+        <is>
+          <t>ZLO03 Mengen und Materialien: Test und Transport</t>
+        </is>
+      </c>
+      <c r="C38" s="21" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="D38" s="16" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="E38" s="18" t="inlineStr">
+        <is>
+          <t>14.08.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="B39" s="16" t="inlineStr">
+        <is>
+          <t>ZC12 Nullmengen: Fehlersuche einschalten</t>
+        </is>
+      </c>
+      <c r="C39" s="21" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="D39" s="16" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="E39" s="18" t="inlineStr">
+        <is>
+          <t>07.09.2026</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="B40" s="16" t="inlineStr">
         <is>
-          <t>Umsatz-Gesamtsicht aller Standorte</t>
+          <t>ZRL2 Mengenrabatt Trafag AT</t>
         </is>
       </c>
       <c r="C40" s="17" t="inlineStr">
@@ -1148,152 +1152,180 @@
       <c r="D40" s="16" t="inlineStr"/>
       <c r="E40" s="18" t="inlineStr">
         <is>
+          <t>30.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>Railway</t>
+        </is>
+      </c>
+      <c r="C42" s="15" t="n"/>
+      <c r="D42" s="15" t="n"/>
+      <c r="E42" s="15" t="n"/>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="B43" s="16" t="inlineStr">
+        <is>
+          <t>Umsatz-Gesamtsicht aller Standorte</t>
+        </is>
+      </c>
+      <c r="C43" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D43" s="16" t="inlineStr"/>
+      <c r="E43" s="18" t="inlineStr">
+        <is>
           <t>29.09.2026</t>
         </is>
       </c>
-    </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="B41" s="16" t="inlineStr">
-        <is>
-          <t>Top-15-Kunden und Schweiz bestätigen</t>
-        </is>
-      </c>
-      <c r="C41" s="19" t="inlineStr">
-        <is>
-          <t>Wartet</t>
-        </is>
-      </c>
-      <c r="D41" s="16" t="inlineStr">
-        <is>
-          <t>Andreas / Patrik</t>
-        </is>
-      </c>
-      <c r="E41" s="18" t="inlineStr">
-        <is>
-          <t>29.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="22" customHeight="1">
-      <c r="B43" s="14" t="inlineStr">
-        <is>
-          <t>Plattform</t>
-        </is>
-      </c>
-      <c r="C43" s="15" t="n"/>
-      <c r="D43" s="15" t="n"/>
-      <c r="E43" s="15" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="B44" s="16" t="inlineStr">
         <is>
-          <t>Webapp schneller</t>
-        </is>
-      </c>
-      <c r="C44" s="17" t="inlineStr">
-        <is>
-          <t>Bereit</t>
-        </is>
-      </c>
-      <c r="D44" s="16" t="inlineStr"/>
+          <t>Top-15-Kunden und Schweiz bestätigen</t>
+        </is>
+      </c>
+      <c r="C44" s="19" t="inlineStr">
+        <is>
+          <t>Wartet</t>
+        </is>
+      </c>
+      <c r="D44" s="16" t="inlineStr">
+        <is>
+          <t>Andreas / Patrik</t>
+        </is>
+      </c>
       <c r="E44" s="18" t="inlineStr">
         <is>
-          <t>28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="20" customHeight="1">
-      <c r="B45" s="16" t="inlineStr">
-        <is>
-          <t>Netzwerk-Reiter: Netzkarte, Verfügbarkeit, Netz oder Daten, Sicherheit</t>
-        </is>
-      </c>
-      <c r="C45" s="17" t="inlineStr">
-        <is>
-          <t>Bereit</t>
-        </is>
-      </c>
-      <c r="D45" s="16" t="inlineStr"/>
-      <c r="E45" s="18" t="inlineStr">
-        <is>
-          <t>02.10.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="B46" s="16" t="inlineStr">
-        <is>
-          <t>AD-Computerkonten im Netzwerk-Reiter einschalten</t>
-        </is>
-      </c>
-      <c r="C46" s="22" t="inlineStr">
-        <is>
-          <t>Erledigt</t>
-        </is>
-      </c>
-      <c r="D46" s="16" t="inlineStr"/>
-      <c r="E46" s="18" t="inlineStr">
-        <is>
-          <t>02.10.2026</t>
-        </is>
-      </c>
+          <t>29.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="B46" s="14" t="inlineStr">
+        <is>
+          <t>Plattform</t>
+        </is>
+      </c>
+      <c r="C46" s="15" t="n"/>
+      <c r="D46" s="15" t="n"/>
+      <c r="E46" s="15" t="n"/>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="B47" s="16" t="inlineStr">
         <is>
-          <t>Server im Dauerbetrieb</t>
-        </is>
-      </c>
-      <c r="C47" s="19" t="inlineStr">
-        <is>
-          <t>Wartet</t>
-        </is>
-      </c>
-      <c r="D47" s="16" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
+          <t>Webapp schneller</t>
+        </is>
+      </c>
+      <c r="C47" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D47" s="16" t="inlineStr"/>
       <c r="E47" s="18" t="inlineStr">
         <is>
           <t>28.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="22" customHeight="1">
-      <c r="B49" s="14" t="inlineStr">
-        <is>
-          <t>Projekte</t>
-        </is>
-      </c>
-      <c r="C49" s="15" t="n"/>
-      <c r="D49" s="15" t="n"/>
-      <c r="E49" s="15" t="n"/>
+    <row r="48" ht="20" customHeight="1">
+      <c r="B48" s="16" t="inlineStr">
+        <is>
+          <t>Netzwerk-Reiter: Netzkarte, Verfügbarkeit, Netz oder Daten, Sicherheit</t>
+        </is>
+      </c>
+      <c r="C48" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D48" s="16" t="inlineStr"/>
+      <c r="E48" s="18" t="inlineStr">
+        <is>
+          <t>02.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="B49" s="16" t="inlineStr">
+        <is>
+          <t>AD-Computerkonten im Netzwerk-Reiter einschalten</t>
+        </is>
+      </c>
+      <c r="C49" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D49" s="16" t="inlineStr"/>
+      <c r="E49" s="18" t="inlineStr">
+        <is>
+          <t>02.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="20" customHeight="1">
       <c r="B50" s="16" t="inlineStr">
         <is>
+          <t>Server im Dauerbetrieb</t>
+        </is>
+      </c>
+      <c r="C50" s="19" t="inlineStr">
+        <is>
+          <t>Wartet</t>
+        </is>
+      </c>
+      <c r="D50" s="16" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="E50" s="18" t="inlineStr">
+        <is>
+          <t>28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="B52" s="14" t="inlineStr">
+        <is>
+          <t>Projekte</t>
+        </is>
+      </c>
+      <c r="C52" s="15" t="n"/>
+      <c r="D52" s="15" t="n"/>
+      <c r="E52" s="15" t="n"/>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="B53" s="16" t="inlineStr">
+        <is>
           <t>Smartsheet-Ablösung, Power-BI-Verantwortliche, Data Lake</t>
         </is>
       </c>
-      <c r="C50" s="21" t="inlineStr">
+      <c r="C53" s="21" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="D50" s="16" t="inlineStr">
+      <c r="D53" s="16" t="inlineStr">
         <is>
           <t>noch nicht gestartet</t>
         </is>
       </c>
-      <c r="E50" s="18" t="inlineStr">
+      <c r="E53" s="18" t="inlineStr">
         <is>
           <t>29.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="26" customHeight="1">
-      <c r="B52" s="23" t="inlineStr">
+    <row r="55" ht="26" customHeight="1">
+      <c r="B55" s="23" t="inlineStr">
         <is>
           <t>Bereit = erledigt und in Betrieb · Läuft = in Arbeit · Wartet = braucht eine andere Person · Offen = noch nicht begonnen oder Entscheid von Ingo. Details und Nachweise: Wochen_Todo.xlsx.</t>
         </is>
@@ -1302,7 +1334,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B52:E52"/>
+    <mergeCell ref="B55:E55"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Document the Controlling sub-tab, its open questions and the 08:18 deploy
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -594,7 +594,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Stand 02.10.2026  ·  Ingo Kohler</t>
+          <t>Stand 05.10.2026  ·  Ingo Kohler</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 47 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 16 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 19.</t>
+          <t>Hinter dieser Seite stehen 48 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 16 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 19.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document Logistik live state (P76 import of T76K912662 with warning, MES answer), learnings of the day, Wochen_Todo and Status_kurz
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -195,10 +195,10 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -603,7 +603,7 @@
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="B4" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C4" s="5" t="n">
         <v>2</v>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 48 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 16 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 19.</t>
+          <t>Hinter dieser Seite stehen 49 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 16 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 19.</t>
         </is>
       </c>
     </row>
@@ -1007,18 +1007,22 @@
     <row r="32" ht="20" customHeight="1">
       <c r="B32" s="16" t="inlineStr">
         <is>
-          <t>Logistik live: Kommissionierung und Produktion fast in Echtzeit</t>
-        </is>
-      </c>
-      <c r="C32" s="17" t="inlineStr">
-        <is>
-          <t>Bereit</t>
-        </is>
-      </c>
-      <c r="D32" s="16" t="inlineStr"/>
+          <t>Logistik live: Kommissionierung, Produktion, 3D-Lager, Produktivität, Kapazität</t>
+        </is>
+      </c>
+      <c r="C32" s="21" t="inlineStr">
+        <is>
+          <t>Bereit, Ausbau 05.10. produktiv</t>
+        </is>
+      </c>
+      <c r="D32" s="16" t="inlineStr">
+        <is>
+          <t>Import T76K912662 prüfen, Passwort für Namen</t>
+        </is>
+      </c>
       <c r="E32" s="18" t="inlineStr">
         <is>
-          <t>01.10.2026</t>
+          <t>05.10.2026</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1050,7 @@
           <t>Zwei kleine Entscheide (Beschriftung, SAP-Schlüssel)</t>
         </is>
       </c>
-      <c r="C34" s="21" t="inlineStr">
+      <c r="C34" s="22" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
@@ -1100,7 +1104,7 @@
           <t>ZLO03 Mengen und Materialien: Test und Transport</t>
         </is>
       </c>
-      <c r="C38" s="21" t="inlineStr">
+      <c r="C38" s="22" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
@@ -1122,7 +1126,7 @@
           <t>ZC12 Nullmengen: Fehlersuche einschalten</t>
         </is>
       </c>
-      <c r="C39" s="21" t="inlineStr">
+      <c r="C39" s="22" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
@@ -1258,7 +1262,7 @@
           <t>AD-Computerkonten im Netzwerk-Reiter einschalten</t>
         </is>
       </c>
-      <c r="C49" s="22" t="inlineStr">
+      <c r="C49" s="21" t="inlineStr">
         <is>
           <t>Erledigt</t>
         </is>
@@ -1308,7 +1312,7 @@
           <t>Smartsheet-Ablösung, Power-BI-Verantwortliche, Data Lake</t>
         </is>
       </c>
-      <c r="C53" s="21" t="inlineStr">
+      <c r="C53" s="22" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>

</xml_diff>

<commit_message>
Docs: review corrections recorded in Weltlage, Verkauf, Controlling, Netzwerk, Logistik docs; RAG Purchasing/Architecture; Wochen_Todo and Status_kurz with manual and open follow-ups
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -569,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -594,7 +594,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Stand 05.10.2026  ·  Ingo Kohler</t>
+          <t>Stand 06.10.2026  ·  Ingo Kohler</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -609,7 +609,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E4" s="7" t="n">
         <v>4</v>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 49 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 16 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 19.</t>
+          <t>Hinter dieser Seite stehen 50 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 16 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 20.</t>
         </is>
       </c>
     </row>
@@ -1066,64 +1066,64 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="B36" s="14" t="inlineStr">
+    <row r="35" ht="20" customHeight="1">
+      <c r="B35" s="16" t="inlineStr">
+        <is>
+          <t>Einkauf über offenen Bestellwert nach Elikz-Fix informieren</t>
+        </is>
+      </c>
+      <c r="C35" s="19" t="inlineStr">
+        <is>
+          <t>Wartet</t>
+        </is>
+      </c>
+      <c r="D35" s="16" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="E35" s="18" t="inlineStr">
+        <is>
+          <t>06.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="B37" s="14" t="inlineStr">
         <is>
           <t>SAP</t>
         </is>
       </c>
-      <c r="C36" s="15" t="n"/>
-      <c r="D36" s="15" t="n"/>
-      <c r="E36" s="15" t="n"/>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="B37" s="16" t="inlineStr">
-        <is>
-          <t>ZZPRDAT Produktionsdatum: gemeinsamer Test</t>
-        </is>
-      </c>
-      <c r="C37" s="20" t="inlineStr">
-        <is>
-          <t>Läuft</t>
-        </is>
-      </c>
-      <c r="D37" s="16" t="inlineStr">
-        <is>
-          <t>Test 12.10. (Lucas, Marco, Adil)</t>
-        </is>
-      </c>
-      <c r="E37" s="18" t="inlineStr">
-        <is>
-          <t>01.10.2026</t>
-        </is>
-      </c>
+      <c r="C37" s="15" t="n"/>
+      <c r="D37" s="15" t="n"/>
+      <c r="E37" s="15" t="n"/>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="B38" s="16" t="inlineStr">
         <is>
-          <t>ZLO03 Mengen und Materialien: Test und Transport</t>
-        </is>
-      </c>
-      <c r="C38" s="22" t="inlineStr">
-        <is>
-          <t>Offen</t>
+          <t>ZZPRDAT Produktionsdatum: gemeinsamer Test</t>
+        </is>
+      </c>
+      <c r="C38" s="20" t="inlineStr">
+        <is>
+          <t>Läuft</t>
         </is>
       </c>
       <c r="D38" s="16" t="inlineStr">
         <is>
-          <t>Ingo</t>
+          <t>Test 12.10. (Lucas, Marco, Adil)</t>
         </is>
       </c>
       <c r="E38" s="18" t="inlineStr">
         <is>
-          <t>14.08.2026</t>
+          <t>01.10.2026</t>
         </is>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="B39" s="16" t="inlineStr">
         <is>
-          <t>ZC12 Nullmengen: Fehlersuche einschalten</t>
+          <t>ZLO03 Mengen und Materialien: Test und Transport</t>
         </is>
       </c>
       <c r="C39" s="22" t="inlineStr">
@@ -1138,110 +1138,114 @@
       </c>
       <c r="E39" s="18" t="inlineStr">
         <is>
-          <t>07.09.2026</t>
+          <t>14.08.2026</t>
         </is>
       </c>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="B40" s="16" t="inlineStr">
         <is>
+          <t>ZC12 Nullmengen: Fehlersuche einschalten</t>
+        </is>
+      </c>
+      <c r="C40" s="22" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="D40" s="16" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="E40" s="18" t="inlineStr">
+        <is>
+          <t>07.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="B41" s="16" t="inlineStr">
+        <is>
           <t>ZRL2 Mengenrabatt Trafag AT</t>
         </is>
       </c>
-      <c r="C40" s="17" t="inlineStr">
+      <c r="C41" s="17" t="inlineStr">
         <is>
           <t>Bereit</t>
         </is>
       </c>
-      <c r="D40" s="16" t="inlineStr"/>
-      <c r="E40" s="18" t="inlineStr">
+      <c r="D41" s="16" t="inlineStr"/>
+      <c r="E41" s="18" t="inlineStr">
         <is>
           <t>30.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="22" customHeight="1">
-      <c r="B42" s="14" t="inlineStr">
+    <row r="43" ht="22" customHeight="1">
+      <c r="B43" s="14" t="inlineStr">
         <is>
           <t>Railway</t>
         </is>
       </c>
-      <c r="C42" s="15" t="n"/>
-      <c r="D42" s="15" t="n"/>
-      <c r="E42" s="15" t="n"/>
-    </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="B43" s="16" t="inlineStr">
-        <is>
-          <t>Umsatz-Gesamtsicht aller Standorte</t>
-        </is>
-      </c>
-      <c r="C43" s="17" t="inlineStr">
-        <is>
-          <t>Bereit</t>
-        </is>
-      </c>
-      <c r="D43" s="16" t="inlineStr"/>
-      <c r="E43" s="18" t="inlineStr">
-        <is>
-          <t>29.09.2026</t>
-        </is>
-      </c>
+      <c r="C43" s="15" t="n"/>
+      <c r="D43" s="15" t="n"/>
+      <c r="E43" s="15" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="B44" s="16" t="inlineStr">
         <is>
+          <t>Umsatz-Gesamtsicht aller Standorte</t>
+        </is>
+      </c>
+      <c r="C44" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D44" s="16" t="inlineStr"/>
+      <c r="E44" s="18" t="inlineStr">
+        <is>
+          <t>29.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="B45" s="16" t="inlineStr">
+        <is>
           <t>Top-15-Kunden und Schweiz bestätigen</t>
         </is>
       </c>
-      <c r="C44" s="19" t="inlineStr">
+      <c r="C45" s="19" t="inlineStr">
         <is>
           <t>Wartet</t>
         </is>
       </c>
-      <c r="D44" s="16" t="inlineStr">
+      <c r="D45" s="16" t="inlineStr">
         <is>
           <t>Andreas / Patrik</t>
         </is>
       </c>
-      <c r="E44" s="18" t="inlineStr">
+      <c r="E45" s="18" t="inlineStr">
         <is>
           <t>29.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="22" customHeight="1">
-      <c r="B46" s="14" t="inlineStr">
+    <row r="47" ht="22" customHeight="1">
+      <c r="B47" s="14" t="inlineStr">
         <is>
           <t>Plattform</t>
         </is>
       </c>
-      <c r="C46" s="15" t="n"/>
-      <c r="D46" s="15" t="n"/>
-      <c r="E46" s="15" t="n"/>
-    </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="B47" s="16" t="inlineStr">
-        <is>
-          <t>Webapp schneller</t>
-        </is>
-      </c>
-      <c r="C47" s="17" t="inlineStr">
-        <is>
-          <t>Bereit</t>
-        </is>
-      </c>
-      <c r="D47" s="16" t="inlineStr"/>
-      <c r="E47" s="18" t="inlineStr">
-        <is>
-          <t>28.09.2026</t>
-        </is>
-      </c>
+      <c r="C47" s="15" t="n"/>
+      <c r="D47" s="15" t="n"/>
+      <c r="E47" s="15" t="n"/>
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="B48" s="16" t="inlineStr">
         <is>
-          <t>Netzwerk-Reiter: Netzkarte, Verfügbarkeit, Netz oder Daten, Sicherheit</t>
+          <t>Webapp schneller</t>
         </is>
       </c>
       <c r="C48" s="17" t="inlineStr">
@@ -1252,19 +1256,19 @@
       <c r="D48" s="16" t="inlineStr"/>
       <c r="E48" s="18" t="inlineStr">
         <is>
-          <t>02.10.2026</t>
+          <t>28.09.2026</t>
         </is>
       </c>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="B49" s="16" t="inlineStr">
         <is>
-          <t>AD-Computerkonten im Netzwerk-Reiter einschalten</t>
-        </is>
-      </c>
-      <c r="C49" s="21" t="inlineStr">
-        <is>
-          <t>Erledigt</t>
+          <t>Netzwerk-Reiter: Netzkarte, Verfügbarkeit, Netz oder Daten, Sicherheit</t>
+        </is>
+      </c>
+      <c r="C49" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr"/>
@@ -1277,59 +1281,109 @@
     <row r="50" ht="20" customHeight="1">
       <c r="B50" s="16" t="inlineStr">
         <is>
+          <t>AD-Computerkonten im Netzwerk-Reiter einschalten</t>
+        </is>
+      </c>
+      <c r="C50" s="21" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D50" s="16" t="inlineStr"/>
+      <c r="E50" s="18" t="inlineStr">
+        <is>
+          <t>02.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="B51" s="16" t="inlineStr">
+        <is>
           <t>Server im Dauerbetrieb</t>
         </is>
       </c>
-      <c r="C50" s="19" t="inlineStr">
+      <c r="C51" s="19" t="inlineStr">
         <is>
           <t>Wartet</t>
         </is>
       </c>
-      <c r="D50" s="16" t="inlineStr">
+      <c r="D51" s="16" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="E50" s="18" t="inlineStr">
+      <c r="E51" s="18" t="inlineStr">
         <is>
           <t>28.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="22" customHeight="1">
-      <c r="B52" s="14" t="inlineStr">
+    <row r="53" ht="22" customHeight="1">
+      <c r="B53" s="14" t="inlineStr">
         <is>
           <t>Projekte</t>
         </is>
       </c>
-      <c r="C52" s="15" t="n"/>
-      <c r="D52" s="15" t="n"/>
-      <c r="E52" s="15" t="n"/>
-    </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="B53" s="16" t="inlineStr">
+      <c r="C53" s="15" t="n"/>
+      <c r="D53" s="15" t="n"/>
+      <c r="E53" s="15" t="n"/>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="B54" s="16" t="inlineStr">
         <is>
           <t>Smartsheet-Ablösung, Power-BI-Verantwortliche, Data Lake</t>
         </is>
       </c>
-      <c r="C53" s="22" t="inlineStr">
+      <c r="C54" s="22" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="D53" s="16" t="inlineStr">
+      <c r="D54" s="16" t="inlineStr">
         <is>
           <t>noch nicht gestartet</t>
         </is>
       </c>
-      <c r="E53" s="18" t="inlineStr">
+      <c r="E54" s="18" t="inlineStr">
         <is>
           <t>29.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="26" customHeight="1">
-      <c r="B55" s="23" t="inlineStr">
+    <row r="56" ht="22" customHeight="1">
+      <c r="B56" s="14" t="inlineStr">
+        <is>
+          <t>Logistik</t>
+        </is>
+      </c>
+      <c r="C56" s="15" t="n"/>
+      <c r="D56" s="15" t="n"/>
+      <c r="E56" s="15" t="n"/>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="B57" s="16" t="inlineStr">
+        <is>
+          <t>ABAP-Transport Prüfbefund Logistik live (Warenausgangszeit, Kapazität)</t>
+        </is>
+      </c>
+      <c r="C57" s="19" t="inlineStr">
+        <is>
+          <t>Wartet</t>
+        </is>
+      </c>
+      <c r="D57" s="16" t="inlineStr">
+        <is>
+          <t>SE11-Prüfung KBED, T76-Transport</t>
+        </is>
+      </c>
+      <c r="E57" s="18" t="inlineStr">
+        <is>
+          <t>05.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="26" customHeight="1">
+      <c r="B59" s="23" t="inlineStr">
         <is>
           <t>Bereit = erledigt und in Betrieb · Läuft = in Arbeit · Wartet = braucht eine andere Person · Offen = noch nicht begonnen oder Entscheid von Ingo. Details und Nachweise: Wochen_Todo.xlsx.</t>
         </is>
@@ -1338,7 +1392,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B55:E55"/>
+    <mergeCell ref="B59:E59"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Docs: one-stage cost logic, supplier recognition, measured gaps (ISS-007.4), todos and status
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -569,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -594,7 +594,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Stand 06.10.2026  ·  Ingo Kohler</t>
+          <t>Stand 07.10.2026  ·  Ingo Kohler</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -609,7 +609,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E4" s="7" t="n">
         <v>4</v>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 50 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 16 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 20.</t>
+          <t>Hinter dieser Seite stehen 57 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 19 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 20.</t>
         </is>
       </c>
     </row>
@@ -782,88 +782,96 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="B17" s="14" t="inlineStr">
+    <row r="16" ht="20" customHeight="1">
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>TR IT verkauft Indien-Ware ohne Konzernkosten TR IN (Sachnummer fehlt, ISS-007.4)</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>Wartet</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>Prüfung B1-Artikelstamm TR IT</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>07.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Kostenwährung zum Budget- oder Tageskurs</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>Wartet</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Andreas</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="inlineStr">
+        <is>
+          <t>07.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="B19" s="14" t="inlineStr">
         <is>
           <t>Verkauf</t>
         </is>
       </c>
-      <c r="C17" s="15" t="n"/>
-      <c r="D17" s="15" t="n"/>
-      <c r="E17" s="15" t="n"/>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="B18" s="16" t="inlineStr">
+      <c r="C19" s="15" t="n"/>
+      <c r="D19" s="15" t="n"/>
+      <c r="E19" s="15" t="n"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="B20" s="16" t="inlineStr">
         <is>
           <t>Reiter Verkauf: Kunden, Rückgang, Konzentration, Cross-Selling, Preise, Prognose, Weltkarte</t>
         </is>
       </c>
-      <c r="C18" s="17" t="inlineStr">
+      <c r="C20" s="17" t="inlineStr">
         <is>
           <t>Bereit</t>
         </is>
       </c>
-      <c r="D18" s="16" t="inlineStr">
+      <c r="D20" s="16" t="inlineStr">
         <is>
           <t>Sichtprüfung Ingo</t>
         </is>
       </c>
-      <c r="E18" s="18" t="inlineStr">
+      <c r="E20" s="18" t="inlineStr">
         <is>
           <t>02.10.2026</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="B20" s="14" t="inlineStr">
+    <row r="22" ht="22" customHeight="1">
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="C20" s="15" t="n"/>
-      <c r="D20" s="15" t="n"/>
-      <c r="E20" s="15" t="n"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="B21" s="16" t="inlineStr">
-        <is>
-          <t>Kader 8,1 h, übrige 8,0 h je Arbeitstag</t>
-        </is>
-      </c>
-      <c r="C21" s="17" t="inlineStr">
-        <is>
-          <t>Bereit</t>
-        </is>
-      </c>
-      <c r="D21" s="16" t="inlineStr"/>
-      <c r="E21" s="18" t="inlineStr">
-        <is>
-          <t>01.10.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="B22" s="16" t="inlineStr">
-        <is>
-          <t>Abwesenheiten mit Von/Bis, nur genehmigte, Krankenquote je Zeitraum</t>
-        </is>
-      </c>
-      <c r="C22" s="17" t="inlineStr">
-        <is>
-          <t>Bereit</t>
-        </is>
-      </c>
-      <c r="D22" s="16" t="inlineStr"/>
-      <c r="E22" s="18" t="inlineStr">
-        <is>
-          <t>01.10.2026</t>
-        </is>
-      </c>
+      <c r="C22" s="15" t="n"/>
+      <c r="D22" s="15" t="n"/>
+      <c r="E22" s="15" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="B23" s="16" t="inlineStr">
         <is>
-          <t>Absenz-Ampel: bis 4,99 % gelb, ab 5 % rot</t>
+          <t>Kader 8,1 h, übrige 8,0 h je Arbeitstag</t>
         </is>
       </c>
       <c r="C23" s="17" t="inlineStr">
@@ -881,7 +889,7 @@
     <row r="24" ht="20" customHeight="1">
       <c r="B24" s="16" t="inlineStr">
         <is>
-          <t>SAP-Daten täglich automatisch</t>
+          <t>Abwesenheiten mit Von/Bis, nur genehmigte, Krankenquote je Zeitraum</t>
         </is>
       </c>
       <c r="C24" s="17" t="inlineStr">
@@ -899,97 +907,97 @@
     <row r="25" ht="20" customHeight="1">
       <c r="B25" s="16" t="inlineStr">
         <is>
-          <t>Rexx-Berichte täglich automatisch</t>
-        </is>
-      </c>
-      <c r="C25" s="19" t="inlineStr">
-        <is>
-          <t>Wartet</t>
-        </is>
-      </c>
-      <c r="D25" s="16" t="inlineStr">
-        <is>
-          <t>Upgreat</t>
-        </is>
-      </c>
+          <t>Absenz-Ampel: bis 4,99 % gelb, ab 5 % rot</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="18" t="inlineStr">
         <is>
-          <t>30.09.2026</t>
+          <t>01.10.2026</t>
         </is>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="B26" s="16" t="inlineStr">
         <is>
+          <t>SAP-Daten täglich automatisch</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D26" s="16" t="inlineStr"/>
+      <c r="E26" s="18" t="inlineStr">
+        <is>
+          <t>01.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>Rexx-Berichte täglich automatisch</t>
+        </is>
+      </c>
+      <c r="C27" s="19" t="inlineStr">
+        <is>
+          <t>Wartet</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>Upgreat</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>30.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="B28" s="16" t="inlineStr">
+        <is>
           <t>Krankheitsarten bestätigen</t>
         </is>
       </c>
-      <c r="C26" s="19" t="inlineStr">
+      <c r="C28" s="19" t="inlineStr">
         <is>
           <t>Wartet</t>
         </is>
       </c>
-      <c r="D26" s="16" t="inlineStr">
+      <c r="D28" s="16" t="inlineStr">
         <is>
           <t>Sonja</t>
         </is>
       </c>
-      <c r="E26" s="18" t="inlineStr">
+      <c r="E28" s="18" t="inlineStr">
         <is>
           <t>01.10.2026</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="B28" s="14" t="inlineStr">
+    <row r="30" ht="22" customHeight="1">
+      <c r="B30" s="14" t="inlineStr">
         <is>
           <t>Einkauf</t>
         </is>
       </c>
-      <c r="C28" s="15" t="n"/>
-      <c r="D28" s="15" t="n"/>
-      <c r="E28" s="15" t="n"/>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="B29" s="16" t="inlineStr">
-        <is>
-          <t>Seite nach dem Auffrischen sofort da</t>
-        </is>
-      </c>
-      <c r="C29" s="17" t="inlineStr">
-        <is>
-          <t>Bereit</t>
-        </is>
-      </c>
-      <c r="D29" s="16" t="inlineStr"/>
-      <c r="E29" s="18" t="inlineStr">
-        <is>
-          <t>01.10.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="B30" s="16" t="inlineStr">
-        <is>
-          <t>Lagerwert-Verlauf je Woche</t>
-        </is>
-      </c>
-      <c r="C30" s="17" t="inlineStr">
-        <is>
-          <t>Bereit</t>
-        </is>
-      </c>
-      <c r="D30" s="16" t="inlineStr"/>
-      <c r="E30" s="18" t="inlineStr">
-        <is>
-          <t>28.09.2026</t>
-        </is>
-      </c>
+      <c r="C30" s="15" t="n"/>
+      <c r="D30" s="15" t="n"/>
+      <c r="E30" s="15" t="n"/>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="B31" s="16" t="inlineStr">
         <is>
-          <t>Texte Produktgruppen D1/D5</t>
+          <t>Seite nach dem Auffrischen sofort da</t>
         </is>
       </c>
       <c r="C31" s="17" t="inlineStr">
@@ -1007,29 +1015,25 @@
     <row r="32" ht="20" customHeight="1">
       <c r="B32" s="16" t="inlineStr">
         <is>
-          <t>Logistik live: Kommissionierung, Produktion, 3D-Lager, Produktivität, Kapazität</t>
-        </is>
-      </c>
-      <c r="C32" s="21" t="inlineStr">
-        <is>
-          <t>Bereit, Ausbau 05.10. produktiv</t>
-        </is>
-      </c>
-      <c r="D32" s="16" t="inlineStr">
-        <is>
-          <t>Passwort für Namen (Ingo)</t>
-        </is>
-      </c>
+          <t>Lagerwert-Verlauf je Woche</t>
+        </is>
+      </c>
+      <c r="C32" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D32" s="16" t="inlineStr"/>
       <c r="E32" s="18" t="inlineStr">
         <is>
-          <t>05.10.2026</t>
+          <t>28.09.2026</t>
         </is>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="B33" s="16" t="inlineStr">
         <is>
-          <t>Stückliste: Verwendung &amp; Risiko über mehrere Stufen</t>
+          <t>Texte Produktgruppen D1/D5</t>
         </is>
       </c>
       <c r="C33" s="17" t="inlineStr">
@@ -1047,343 +1051,383 @@
     <row r="34" ht="20" customHeight="1">
       <c r="B34" s="16" t="inlineStr">
         <is>
-          <t>Zwei kleine Entscheide (Beschriftung, SAP-Schlüssel)</t>
-        </is>
-      </c>
-      <c r="C34" s="22" t="inlineStr">
-        <is>
-          <t>Offen</t>
+          <t>Logistik live: Kommissionierung, Produktion, 3D-Lager, Produktivität, Kapazität</t>
+        </is>
+      </c>
+      <c r="C34" s="21" t="inlineStr">
+        <is>
+          <t>Bereit, Ausbau 05.10. produktiv</t>
         </is>
       </c>
       <c r="D34" s="16" t="inlineStr">
         <is>
-          <t>Ingo</t>
+          <t>Passwort für Namen (Ingo)</t>
         </is>
       </c>
       <c r="E34" s="18" t="inlineStr">
         <is>
-          <t>29.09.2026</t>
+          <t>05.10.2026</t>
         </is>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="B35" s="16" t="inlineStr">
         <is>
+          <t>Stückliste: Verwendung &amp; Risiko über mehrere Stufen</t>
+        </is>
+      </c>
+      <c r="C35" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D35" s="16" t="inlineStr"/>
+      <c r="E35" s="18" t="inlineStr">
+        <is>
+          <t>01.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="B36" s="16" t="inlineStr">
+        <is>
+          <t>Zwei kleine Entscheide (Beschriftung, SAP-Schlüssel)</t>
+        </is>
+      </c>
+      <c r="C36" s="22" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="D36" s="16" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="E36" s="18" t="inlineStr">
+        <is>
+          <t>29.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="B37" s="16" t="inlineStr">
+        <is>
           <t>Einkauf über offenen Bestellwert nach Elikz-Fix informieren</t>
         </is>
       </c>
-      <c r="C35" s="19" t="inlineStr">
+      <c r="C37" s="19" t="inlineStr">
         <is>
           <t>Wartet</t>
         </is>
       </c>
-      <c r="D35" s="16" t="inlineStr">
+      <c r="D37" s="16" t="inlineStr">
         <is>
           <t>Ingo</t>
         </is>
       </c>
-      <c r="E35" s="18" t="inlineStr">
+      <c r="E37" s="18" t="inlineStr">
         <is>
           <t>06.10.2026</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="22" customHeight="1">
-      <c r="B37" s="14" t="inlineStr">
+    <row r="39" ht="22" customHeight="1">
+      <c r="B39" s="14" t="inlineStr">
         <is>
           <t>SAP</t>
         </is>
       </c>
-      <c r="C37" s="15" t="n"/>
-      <c r="D37" s="15" t="n"/>
-      <c r="E37" s="15" t="n"/>
-    </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="B38" s="16" t="inlineStr">
-        <is>
-          <t>ZZPRDAT Produktionsdatum: gemeinsamer Test</t>
-        </is>
-      </c>
-      <c r="C38" s="20" t="inlineStr">
-        <is>
-          <t>Läuft</t>
-        </is>
-      </c>
-      <c r="D38" s="16" t="inlineStr">
-        <is>
-          <t>Test 12.10. (Lucas, Marco, Adil)</t>
-        </is>
-      </c>
-      <c r="E38" s="18" t="inlineStr">
-        <is>
-          <t>01.10.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="B39" s="16" t="inlineStr">
-        <is>
-          <t>ZLO03 Mengen und Materialien: Test und Transport</t>
-        </is>
-      </c>
-      <c r="C39" s="22" t="inlineStr">
-        <is>
-          <t>Offen</t>
-        </is>
-      </c>
-      <c r="D39" s="16" t="inlineStr">
-        <is>
-          <t>Ingo</t>
-        </is>
-      </c>
-      <c r="E39" s="18" t="inlineStr">
-        <is>
-          <t>14.08.2026</t>
-        </is>
-      </c>
+      <c r="C39" s="15" t="n"/>
+      <c r="D39" s="15" t="n"/>
+      <c r="E39" s="15" t="n"/>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="B40" s="16" t="inlineStr">
         <is>
-          <t>ZC12 Nullmengen: Fehlersuche einschalten</t>
-        </is>
-      </c>
-      <c r="C40" s="22" t="inlineStr">
-        <is>
-          <t>Offen</t>
+          <t>ZZPRDAT Produktionsdatum: gemeinsamer Test</t>
+        </is>
+      </c>
+      <c r="C40" s="20" t="inlineStr">
+        <is>
+          <t>Läuft</t>
         </is>
       </c>
       <c r="D40" s="16" t="inlineStr">
         <is>
-          <t>Ingo</t>
+          <t>Test 12.10. (Lucas, Marco, Adil)</t>
         </is>
       </c>
       <c r="E40" s="18" t="inlineStr">
         <is>
-          <t>07.09.2026</t>
+          <t>01.10.2026</t>
         </is>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="B41" s="16" t="inlineStr">
         <is>
+          <t>ZLO03 Mengen und Materialien: Test und Transport</t>
+        </is>
+      </c>
+      <c r="C41" s="22" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="D41" s="16" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="E41" s="18" t="inlineStr">
+        <is>
+          <t>14.08.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="B42" s="16" t="inlineStr">
+        <is>
+          <t>ZC12 Nullmengen: Fehlersuche einschalten</t>
+        </is>
+      </c>
+      <c r="C42" s="22" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="D42" s="16" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="E42" s="18" t="inlineStr">
+        <is>
+          <t>07.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="B43" s="16" t="inlineStr">
+        <is>
           <t>ZRL2 Mengenrabatt Trafag AT</t>
         </is>
       </c>
-      <c r="C41" s="17" t="inlineStr">
+      <c r="C43" s="17" t="inlineStr">
         <is>
           <t>Bereit</t>
         </is>
       </c>
-      <c r="D41" s="16" t="inlineStr"/>
-      <c r="E41" s="18" t="inlineStr">
+      <c r="D43" s="16" t="inlineStr"/>
+      <c r="E43" s="18" t="inlineStr">
         <is>
           <t>30.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="22" customHeight="1">
-      <c r="B43" s="14" t="inlineStr">
+    <row r="45" ht="22" customHeight="1">
+      <c r="B45" s="14" t="inlineStr">
         <is>
           <t>Railway</t>
         </is>
       </c>
-      <c r="C43" s="15" t="n"/>
-      <c r="D43" s="15" t="n"/>
-      <c r="E43" s="15" t="n"/>
-    </row>
-    <row r="44" ht="20" customHeight="1">
-      <c r="B44" s="16" t="inlineStr">
+      <c r="C45" s="15" t="n"/>
+      <c r="D45" s="15" t="n"/>
+      <c r="E45" s="15" t="n"/>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="B46" s="16" t="inlineStr">
         <is>
           <t>Umsatz-Gesamtsicht aller Standorte</t>
         </is>
       </c>
-      <c r="C44" s="17" t="inlineStr">
+      <c r="C46" s="17" t="inlineStr">
         <is>
           <t>Bereit</t>
         </is>
       </c>
-      <c r="D44" s="16" t="inlineStr"/>
-      <c r="E44" s="18" t="inlineStr">
+      <c r="D46" s="16" t="inlineStr"/>
+      <c r="E46" s="18" t="inlineStr">
         <is>
           <t>29.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="20" customHeight="1">
-      <c r="B45" s="16" t="inlineStr">
+    <row r="47" ht="20" customHeight="1">
+      <c r="B47" s="16" t="inlineStr">
         <is>
           <t>Top-15-Kunden und Schweiz bestätigen</t>
         </is>
       </c>
-      <c r="C45" s="19" t="inlineStr">
+      <c r="C47" s="19" t="inlineStr">
         <is>
           <t>Wartet</t>
         </is>
       </c>
-      <c r="D45" s="16" t="inlineStr">
+      <c r="D47" s="16" t="inlineStr">
         <is>
           <t>Andreas / Patrik</t>
         </is>
       </c>
-      <c r="E45" s="18" t="inlineStr">
+      <c r="E47" s="18" t="inlineStr">
         <is>
           <t>29.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="22" customHeight="1">
-      <c r="B47" s="14" t="inlineStr">
+    <row r="49" ht="22" customHeight="1">
+      <c r="B49" s="14" t="inlineStr">
         <is>
           <t>Plattform</t>
         </is>
       </c>
-      <c r="C47" s="15" t="n"/>
-      <c r="D47" s="15" t="n"/>
-      <c r="E47" s="15" t="n"/>
-    </row>
-    <row r="48" ht="20" customHeight="1">
-      <c r="B48" s="16" t="inlineStr">
-        <is>
-          <t>Webapp schneller</t>
-        </is>
-      </c>
-      <c r="C48" s="17" t="inlineStr">
-        <is>
-          <t>Bereit</t>
-        </is>
-      </c>
-      <c r="D48" s="16" t="inlineStr"/>
-      <c r="E48" s="18" t="inlineStr">
-        <is>
-          <t>28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="20" customHeight="1">
-      <c r="B49" s="16" t="inlineStr">
-        <is>
-          <t>Netzwerk-Reiter: Netzkarte, Verfügbarkeit, Netz oder Daten, Sicherheit</t>
-        </is>
-      </c>
-      <c r="C49" s="17" t="inlineStr">
-        <is>
-          <t>Bereit</t>
-        </is>
-      </c>
-      <c r="D49" s="16" t="inlineStr"/>
-      <c r="E49" s="18" t="inlineStr">
-        <is>
-          <t>02.10.2026</t>
-        </is>
-      </c>
+      <c r="C49" s="15" t="n"/>
+      <c r="D49" s="15" t="n"/>
+      <c r="E49" s="15" t="n"/>
     </row>
     <row r="50" ht="20" customHeight="1">
       <c r="B50" s="16" t="inlineStr">
         <is>
-          <t>AD-Computerkonten im Netzwerk-Reiter einschalten</t>
-        </is>
-      </c>
-      <c r="C50" s="21" t="inlineStr">
-        <is>
-          <t>Erledigt</t>
+          <t>Webapp schneller</t>
+        </is>
+      </c>
+      <c r="C50" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
         </is>
       </c>
       <c r="D50" s="16" t="inlineStr"/>
       <c r="E50" s="18" t="inlineStr">
         <is>
-          <t>02.10.2026</t>
+          <t>28.09.2026</t>
         </is>
       </c>
     </row>
     <row r="51" ht="20" customHeight="1">
       <c r="B51" s="16" t="inlineStr">
         <is>
+          <t>Netzwerk-Reiter: Netzkarte, Verfügbarkeit, Netz oder Daten, Sicherheit</t>
+        </is>
+      </c>
+      <c r="C51" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D51" s="16" t="inlineStr"/>
+      <c r="E51" s="18" t="inlineStr">
+        <is>
+          <t>02.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="B52" s="16" t="inlineStr">
+        <is>
+          <t>AD-Computerkonten im Netzwerk-Reiter einschalten</t>
+        </is>
+      </c>
+      <c r="C52" s="21" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D52" s="16" t="inlineStr"/>
+      <c r="E52" s="18" t="inlineStr">
+        <is>
+          <t>02.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="B53" s="16" t="inlineStr">
+        <is>
           <t>Server im Dauerbetrieb</t>
         </is>
       </c>
-      <c r="C51" s="19" t="inlineStr">
+      <c r="C53" s="19" t="inlineStr">
         <is>
           <t>Wartet</t>
         </is>
       </c>
-      <c r="D51" s="16" t="inlineStr">
+      <c r="D53" s="16" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="E51" s="18" t="inlineStr">
+      <c r="E53" s="18" t="inlineStr">
         <is>
           <t>28.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="22" customHeight="1">
-      <c r="B53" s="14" t="inlineStr">
+    <row r="55" ht="22" customHeight="1">
+      <c r="B55" s="14" t="inlineStr">
         <is>
           <t>Projekte</t>
         </is>
       </c>
-      <c r="C53" s="15" t="n"/>
-      <c r="D53" s="15" t="n"/>
-      <c r="E53" s="15" t="n"/>
-    </row>
-    <row r="54" ht="20" customHeight="1">
-      <c r="B54" s="16" t="inlineStr">
+      <c r="C55" s="15" t="n"/>
+      <c r="D55" s="15" t="n"/>
+      <c r="E55" s="15" t="n"/>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="B56" s="16" t="inlineStr">
         <is>
           <t>Smartsheet-Ablösung, Power-BI-Verantwortliche, Data Lake</t>
         </is>
       </c>
-      <c r="C54" s="22" t="inlineStr">
+      <c r="C56" s="22" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="D54" s="16" t="inlineStr">
+      <c r="D56" s="16" t="inlineStr">
         <is>
           <t>noch nicht gestartet</t>
         </is>
       </c>
-      <c r="E54" s="18" t="inlineStr">
+      <c r="E56" s="18" t="inlineStr">
         <is>
           <t>29.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="22" customHeight="1">
-      <c r="B56" s="14" t="inlineStr">
+    <row r="58" ht="22" customHeight="1">
+      <c r="B58" s="14" t="inlineStr">
         <is>
           <t>Logistik</t>
         </is>
       </c>
-      <c r="C56" s="15" t="n"/>
-      <c r="D56" s="15" t="n"/>
-      <c r="E56" s="15" t="n"/>
-    </row>
-    <row r="57" ht="20" customHeight="1">
-      <c r="B57" s="16" t="inlineStr">
+      <c r="C58" s="15" t="n"/>
+      <c r="D58" s="15" t="n"/>
+      <c r="E58" s="15" t="n"/>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="B59" s="16" t="inlineStr">
         <is>
           <t>ABAP-Transport Prüfbefund Logistik live (Warenausgangszeit, Kapazität)</t>
         </is>
       </c>
-      <c r="C57" s="19" t="inlineStr">
+      <c r="C59" s="19" t="inlineStr">
         <is>
           <t>Wartet</t>
         </is>
       </c>
-      <c r="D57" s="16" t="inlineStr">
+      <c r="D59" s="16" t="inlineStr">
         <is>
           <t>SE11-Prüfung KBED, T76-Transport</t>
         </is>
       </c>
-      <c r="E57" s="18" t="inlineStr">
+      <c r="E59" s="18" t="inlineStr">
         <is>
           <t>05.10.2026</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="26" customHeight="1">
-      <c r="B59" s="23" t="inlineStr">
+    <row r="61" ht="26" customHeight="1">
+      <c r="B61" s="23" t="inlineStr">
         <is>
           <t>Bereit = erledigt und in Betrieb · Läuft = in Arbeit · Wartet = braucht eine andere Person · Offen = noch nicht begonnen oder Entscheid von Ingo. Details und Nachweise: Wochen_Todo.xlsx.</t>
         </is>
@@ -1392,7 +1436,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B59:E59"/>
+    <mergeCell ref="B61:E61"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Docs: Status_kurz and LEARNINGS for ZM_OFFENE_FAUF pegging
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -569,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -609,7 +609,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E4" s="7" t="n">
         <v>4</v>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 57 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 19 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 20.</t>
+          <t>Hinter dieser Seite stehen 58 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 19 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 20.</t>
         </is>
       </c>
     </row>
@@ -1426,8 +1426,30 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="26" customHeight="1">
-      <c r="B61" s="23" t="inlineStr">
+    <row r="60" ht="20" customHeight="1">
+      <c r="B60" s="16" t="inlineStr">
+        <is>
+          <t>ZM_OFFENE_FAUF mit Bedarfsverursacher (T76 fertig, Transport T76K912714)</t>
+        </is>
+      </c>
+      <c r="C60" s="19" t="inlineStr">
+        <is>
+          <t>Wartet</t>
+        </is>
+      </c>
+      <c r="D60" s="16" t="inlineStr">
+        <is>
+          <t>Ingo: Sichtung T76, Freigabe, Import P76</t>
+        </is>
+      </c>
+      <c r="E60" s="18" t="inlineStr">
+        <is>
+          <t>07.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="26" customHeight="1">
+      <c r="B62" s="23" t="inlineStr">
         <is>
           <t>Bereit = erledigt und in Betrieb · Läuft = in Arbeit · Wartet = braucht eine andere Person · Offen = noch nicht begonnen oder Entscheid von Ingo. Details und Nachweise: Wochen_Todo.xlsx.</t>
         </is>
@@ -1436,7 +1458,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B61:E61"/>
+    <mergeCell ref="B62:E62"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
New tab Operations (Shopfloor): PPA-Shopfloor app in the Cockpit (frontend kept, Python backend ported to C#), access only for allowed users until production head approves; SAP sync for ZD05 and forecast orders (ShopZd05Set/ShopAufSet, T76K912718), switched off until P76
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -569,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -609,7 +609,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E4" s="7" t="n">
         <v>4</v>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 58 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 19 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 20.</t>
+          <t>Hinter dieser Seite stehen 59 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 19 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 20.</t>
         </is>
       </c>
     </row>
@@ -1362,94 +1362,116 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="22" customHeight="1">
-      <c r="B55" s="14" t="inlineStr">
+    <row r="54" ht="20" customHeight="1">
+      <c r="B54" s="16" t="inlineStr">
+        <is>
+          <t>Operations (Shopfloor): Freigabe Leitung Produktion, P76-Import T76K912718</t>
+        </is>
+      </c>
+      <c r="C54" s="19" t="inlineStr">
+        <is>
+          <t>Wartet</t>
+        </is>
+      </c>
+      <c r="D54" s="16" t="inlineStr">
+        <is>
+          <t>Ingo / Leitung Produktion</t>
+        </is>
+      </c>
+      <c r="E54" s="18" t="inlineStr">
+        <is>
+          <t>07.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="B56" s="14" t="inlineStr">
         <is>
           <t>Projekte</t>
         </is>
       </c>
-      <c r="C55" s="15" t="n"/>
-      <c r="D55" s="15" t="n"/>
-      <c r="E55" s="15" t="n"/>
-    </row>
-    <row r="56" ht="20" customHeight="1">
-      <c r="B56" s="16" t="inlineStr">
+      <c r="C56" s="15" t="n"/>
+      <c r="D56" s="15" t="n"/>
+      <c r="E56" s="15" t="n"/>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="B57" s="16" t="inlineStr">
         <is>
           <t>Smartsheet-Ablösung, Power-BI-Verantwortliche, Data Lake</t>
         </is>
       </c>
-      <c r="C56" s="22" t="inlineStr">
+      <c r="C57" s="22" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="D56" s="16" t="inlineStr">
+      <c r="D57" s="16" t="inlineStr">
         <is>
           <t>noch nicht gestartet</t>
         </is>
       </c>
-      <c r="E56" s="18" t="inlineStr">
+      <c r="E57" s="18" t="inlineStr">
         <is>
           <t>29.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="22" customHeight="1">
-      <c r="B58" s="14" t="inlineStr">
+    <row r="59" ht="22" customHeight="1">
+      <c r="B59" s="14" t="inlineStr">
         <is>
           <t>Logistik</t>
         </is>
       </c>
-      <c r="C58" s="15" t="n"/>
-      <c r="D58" s="15" t="n"/>
-      <c r="E58" s="15" t="n"/>
-    </row>
-    <row r="59" ht="20" customHeight="1">
-      <c r="B59" s="16" t="inlineStr">
-        <is>
-          <t>ABAP-Transport Prüfbefund Logistik live (Warenausgangszeit, Kapazität)</t>
-        </is>
-      </c>
-      <c r="C59" s="19" t="inlineStr">
-        <is>
-          <t>Wartet</t>
-        </is>
-      </c>
-      <c r="D59" s="16" t="inlineStr">
-        <is>
-          <t>SE11-Prüfung KBED, T76-Transport</t>
-        </is>
-      </c>
-      <c r="E59" s="18" t="inlineStr">
-        <is>
-          <t>05.10.2026</t>
-        </is>
-      </c>
+      <c r="C59" s="15" t="n"/>
+      <c r="D59" s="15" t="n"/>
+      <c r="E59" s="15" t="n"/>
     </row>
     <row r="60" ht="20" customHeight="1">
       <c r="B60" s="16" t="inlineStr">
         <is>
+          <t>ABAP-Transport Prüfbefund Logistik live (Warenausgangszeit, Kapazität)</t>
+        </is>
+      </c>
+      <c r="C60" s="19" t="inlineStr">
+        <is>
+          <t>Wartet</t>
+        </is>
+      </c>
+      <c r="D60" s="16" t="inlineStr">
+        <is>
+          <t>SE11-Prüfung KBED, T76-Transport</t>
+        </is>
+      </c>
+      <c r="E60" s="18" t="inlineStr">
+        <is>
+          <t>05.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="B61" s="16" t="inlineStr">
+        <is>
           <t>ZM_OFFENE_FAUF mit Bedarfsverursacher (T76 fertig, Transport T76K912714)</t>
         </is>
       </c>
-      <c r="C60" s="19" t="inlineStr">
+      <c r="C61" s="19" t="inlineStr">
         <is>
           <t>Wartet</t>
         </is>
       </c>
-      <c r="D60" s="16" t="inlineStr">
+      <c r="D61" s="16" t="inlineStr">
         <is>
           <t>Ingo: Sichtung T76, Freigabe, Import P76</t>
         </is>
       </c>
-      <c r="E60" s="18" t="inlineStr">
+      <c r="E61" s="18" t="inlineStr">
         <is>
           <t>07.10.2026</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="26" customHeight="1">
-      <c r="B62" s="23" t="inlineStr">
+    <row r="63" ht="26" customHeight="1">
+      <c r="B63" s="23" t="inlineStr">
         <is>
           <t>Bereit = erledigt und in Betrieb · Läuft = in Arbeit · Wartet = braucht eine andere Person · Offen = noch nicht begonnen oder Entscheid von Ingo. Details und Nachweise: Wochen_Todo.xlsx.</t>
         </is>
@@ -1457,8 +1479,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="B63:E63"/>
     <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B62:E62"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Docs: coordination cleaned up (finished rows and index before 2026-10-02 moved to history), T76K912714 imported to P76 on 2026-10-09
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -594,7 +594,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Stand 08.10.2026  ·  Ingo Kohler</t>
+          <t>Stand 09.10.2026  ·  Ingo Kohler</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -606,10 +606,10 @@
         <v>14</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E4" s="7" t="n">
         <v>4</v>
@@ -1451,22 +1451,22 @@
     <row r="61" ht="20" customHeight="1">
       <c r="B61" s="16" t="inlineStr">
         <is>
-          <t>ZM_OFFENE_FAUF mit Bedarfsverursacher (T76 fertig, Transport T76K912714)</t>
-        </is>
-      </c>
-      <c r="C61" s="19" t="inlineStr">
-        <is>
-          <t>Wartet</t>
+          <t>ZM_OFFENE_FAUF mit Bedarfsverursacher (T76K912714 am 09.10. in P76)</t>
+        </is>
+      </c>
+      <c r="C61" s="20" t="inlineStr">
+        <is>
+          <t>Läuft</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
         <is>
-          <t>Ingo: Sichtung T76, Freigabe, Import P76</t>
+          <t>Fabio: Layout in P76 prüfen, Fall BANF Werk 1200</t>
         </is>
       </c>
       <c r="E61" s="18" t="inlineStr">
         <is>
-          <t>07.10.2026</t>
+          <t>09.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs: Trafag Reddit (doc, manual chapter 9 and Word file, router, baum, architecture, lastchange, todo/status, coordination reservation)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -569,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -606,7 +606,7 @@
         <v>14</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D4" s="6" t="n">
         <v>12</v>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 62 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 19 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 20.</t>
+          <t>Hinter dieser Seite stehen 63 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 19 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 20.</t>
         </is>
       </c>
     </row>
@@ -1384,94 +1384,116 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="22" customHeight="1">
-      <c r="B56" s="14" t="inlineStr">
+    <row r="55" ht="20" customHeight="1">
+      <c r="B55" s="16" t="inlineStr">
+        <is>
+          <t>Trafag Reddit: Forum mit Abstimmung, für alle sichtbar</t>
+        </is>
+      </c>
+      <c r="C55" s="20" t="inlineStr">
+        <is>
+          <t>Läuft</t>
+        </is>
+      </c>
+      <c r="D55" s="16" t="inlineStr">
+        <is>
+          <t>Ingo: Ankündigung entscheiden</t>
+        </is>
+      </c>
+      <c r="E55" s="18" t="inlineStr">
+        <is>
+          <t>09.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="B57" s="14" t="inlineStr">
         <is>
           <t>Projekte</t>
         </is>
       </c>
-      <c r="C56" s="15" t="n"/>
-      <c r="D56" s="15" t="n"/>
-      <c r="E56" s="15" t="n"/>
-    </row>
-    <row r="57" ht="20" customHeight="1">
-      <c r="B57" s="16" t="inlineStr">
+      <c r="C57" s="15" t="n"/>
+      <c r="D57" s="15" t="n"/>
+      <c r="E57" s="15" t="n"/>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="B58" s="16" t="inlineStr">
         <is>
           <t>Smartsheet-Ablösung, Power-BI-Verantwortliche, Data Lake</t>
         </is>
       </c>
-      <c r="C57" s="22" t="inlineStr">
+      <c r="C58" s="22" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="D57" s="16" t="inlineStr">
+      <c r="D58" s="16" t="inlineStr">
         <is>
           <t>noch nicht gestartet</t>
         </is>
       </c>
-      <c r="E57" s="18" t="inlineStr">
+      <c r="E58" s="18" t="inlineStr">
         <is>
           <t>29.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="22" customHeight="1">
-      <c r="B59" s="14" t="inlineStr">
+    <row r="60" ht="22" customHeight="1">
+      <c r="B60" s="14" t="inlineStr">
         <is>
           <t>Logistik</t>
         </is>
       </c>
-      <c r="C59" s="15" t="n"/>
-      <c r="D59" s="15" t="n"/>
-      <c r="E59" s="15" t="n"/>
-    </row>
-    <row r="60" ht="20" customHeight="1">
-      <c r="B60" s="16" t="inlineStr">
-        <is>
-          <t>ABAP-Transport Prüfbefund Logistik live (Warenausgangszeit, Kapazität)</t>
-        </is>
-      </c>
-      <c r="C60" s="19" t="inlineStr">
-        <is>
-          <t>Wartet</t>
-        </is>
-      </c>
-      <c r="D60" s="16" t="inlineStr">
-        <is>
-          <t>SE11-Prüfung KBED, T76-Transport</t>
-        </is>
-      </c>
-      <c r="E60" s="18" t="inlineStr">
-        <is>
-          <t>05.10.2026</t>
-        </is>
-      </c>
+      <c r="C60" s="15" t="n"/>
+      <c r="D60" s="15" t="n"/>
+      <c r="E60" s="15" t="n"/>
     </row>
     <row r="61" ht="20" customHeight="1">
       <c r="B61" s="16" t="inlineStr">
         <is>
+          <t>ABAP-Transport Prüfbefund Logistik live (Warenausgangszeit, Kapazität)</t>
+        </is>
+      </c>
+      <c r="C61" s="19" t="inlineStr">
+        <is>
+          <t>Wartet</t>
+        </is>
+      </c>
+      <c r="D61" s="16" t="inlineStr">
+        <is>
+          <t>SE11-Prüfung KBED, T76-Transport</t>
+        </is>
+      </c>
+      <c r="E61" s="18" t="inlineStr">
+        <is>
+          <t>05.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="B62" s="16" t="inlineStr">
+        <is>
           <t>ZM_OFFENE_FAUF mit Bedarfsverursacher (T76K912714 am 09.10. in P76)</t>
         </is>
       </c>
-      <c r="C61" s="20" t="inlineStr">
+      <c r="C62" s="20" t="inlineStr">
         <is>
           <t>Läuft</t>
         </is>
       </c>
-      <c r="D61" s="16" t="inlineStr">
+      <c r="D62" s="16" t="inlineStr">
         <is>
           <t>Fabio: Layout in P76 prüfen, Fall BANF Werk 1200</t>
         </is>
       </c>
-      <c r="E61" s="18" t="inlineStr">
+      <c r="E62" s="18" t="inlineStr">
         <is>
           <t>09.10.2026</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="26" customHeight="1">
-      <c r="B63" s="23" t="inlineStr">
+    <row r="64" ht="26" customHeight="1">
+      <c r="B64" s="23" t="inlineStr">
         <is>
           <t>Bereit = erledigt und in Betrieb · Läuft = in Arbeit · Wartet = braucht eine andere Person · Offen = noch nicht begonnen oder Entscheid von Ingo. Details und Nachweise: Wochen_Todo.xlsx.</t>
         </is>
@@ -1479,7 +1501,7 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B63:E63"/>
+    <mergeCell ref="B64:E64"/>
     <mergeCell ref="B7:E7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Docs: Trafag Projekte (doc, router, baum, architecture, old project suite marked superseded, lastchange, todo/status, learnings, coordination reservation)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -569,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -606,7 +606,7 @@
         <v>14</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" s="6" t="n">
         <v>12</v>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 63 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 19 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 20.</t>
+          <t>Hinter dieser Seite stehen 64 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 19 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 20.</t>
         </is>
       </c>
     </row>
@@ -1406,94 +1406,116 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="22" customHeight="1">
-      <c r="B57" s="14" t="inlineStr">
+    <row r="56" ht="20" customHeight="1">
+      <c r="B56" s="16" t="inlineStr">
+        <is>
+          <t>Trafag Projekte: Board, Backlog/Sprints, Zeitachse, Kalender, Diagramme</t>
+        </is>
+      </c>
+      <c r="C56" s="20" t="inlineStr">
+        <is>
+          <t>Läuft</t>
+        </is>
+      </c>
+      <c r="D56" s="16" t="inlineStr">
+        <is>
+          <t>Ingo: erstes echtes Projekt anlegen</t>
+        </is>
+      </c>
+      <c r="E56" s="18" t="inlineStr">
+        <is>
+          <t>09.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="22" customHeight="1">
+      <c r="B58" s="14" t="inlineStr">
         <is>
           <t>Projekte</t>
         </is>
       </c>
-      <c r="C57" s="15" t="n"/>
-      <c r="D57" s="15" t="n"/>
-      <c r="E57" s="15" t="n"/>
-    </row>
-    <row r="58" ht="20" customHeight="1">
-      <c r="B58" s="16" t="inlineStr">
+      <c r="C58" s="15" t="n"/>
+      <c r="D58" s="15" t="n"/>
+      <c r="E58" s="15" t="n"/>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="B59" s="16" t="inlineStr">
         <is>
           <t>Smartsheet-Ablösung, Power-BI-Verantwortliche, Data Lake</t>
         </is>
       </c>
-      <c r="C58" s="22" t="inlineStr">
+      <c r="C59" s="22" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="D58" s="16" t="inlineStr">
+      <c r="D59" s="16" t="inlineStr">
         <is>
           <t>noch nicht gestartet</t>
         </is>
       </c>
-      <c r="E58" s="18" t="inlineStr">
+      <c r="E59" s="18" t="inlineStr">
         <is>
           <t>29.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="22" customHeight="1">
-      <c r="B60" s="14" t="inlineStr">
+    <row r="61" ht="22" customHeight="1">
+      <c r="B61" s="14" t="inlineStr">
         <is>
           <t>Logistik</t>
         </is>
       </c>
-      <c r="C60" s="15" t="n"/>
-      <c r="D60" s="15" t="n"/>
-      <c r="E60" s="15" t="n"/>
-    </row>
-    <row r="61" ht="20" customHeight="1">
-      <c r="B61" s="16" t="inlineStr">
-        <is>
-          <t>ABAP-Transport Prüfbefund Logistik live (Warenausgangszeit, Kapazität)</t>
-        </is>
-      </c>
-      <c r="C61" s="19" t="inlineStr">
-        <is>
-          <t>Wartet</t>
-        </is>
-      </c>
-      <c r="D61" s="16" t="inlineStr">
-        <is>
-          <t>SE11-Prüfung KBED, T76-Transport</t>
-        </is>
-      </c>
-      <c r="E61" s="18" t="inlineStr">
-        <is>
-          <t>05.10.2026</t>
-        </is>
-      </c>
+      <c r="C61" s="15" t="n"/>
+      <c r="D61" s="15" t="n"/>
+      <c r="E61" s="15" t="n"/>
     </row>
     <row r="62" ht="20" customHeight="1">
       <c r="B62" s="16" t="inlineStr">
         <is>
+          <t>ABAP-Transport Prüfbefund Logistik live (Warenausgangszeit, Kapazität)</t>
+        </is>
+      </c>
+      <c r="C62" s="19" t="inlineStr">
+        <is>
+          <t>Wartet</t>
+        </is>
+      </c>
+      <c r="D62" s="16" t="inlineStr">
+        <is>
+          <t>SE11-Prüfung KBED, T76-Transport</t>
+        </is>
+      </c>
+      <c r="E62" s="18" t="inlineStr">
+        <is>
+          <t>05.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="20" customHeight="1">
+      <c r="B63" s="16" t="inlineStr">
+        <is>
           <t>ZM_OFFENE_FAUF mit Bedarfsverursacher (T76K912714 am 09.10. in P76)</t>
         </is>
       </c>
-      <c r="C62" s="20" t="inlineStr">
+      <c r="C63" s="20" t="inlineStr">
         <is>
           <t>Läuft</t>
         </is>
       </c>
-      <c r="D62" s="16" t="inlineStr">
+      <c r="D63" s="16" t="inlineStr">
         <is>
           <t>Fabio: Layout in P76 prüfen, Fall BANF Werk 1200</t>
         </is>
       </c>
-      <c r="E62" s="18" t="inlineStr">
+      <c r="E63" s="18" t="inlineStr">
         <is>
           <t>09.10.2026</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="26" customHeight="1">
-      <c r="B64" s="23" t="inlineStr">
+    <row r="65" ht="26" customHeight="1">
+      <c r="B65" s="23" t="inlineStr">
         <is>
           <t>Bereit = erledigt und in Betrieb · Läuft = in Arbeit · Wartet = braucht eine andere Person · Offen = noch nicht begonnen oder Entscheid von Ingo. Details und Nachweise: Wochen_Todo.xlsx.</t>
         </is>
@@ -1501,8 +1523,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B64:E64"/>
     <mergeCell ref="B7:E7"/>
+    <mergeCell ref="B65:E65"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Docs: SAP transports T76K912724/T76K912718 in P76, Shopfloor SAP sync on (first runs 11:33/12:47), contracts and LZ codes loaded (delta 12:27), deploys 11:32 and 12:45, learning on deploy aborting a running delta
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -1365,7 +1365,7 @@
     <row r="54" ht="20" customHeight="1">
       <c r="B54" s="16" t="inlineStr">
         <is>
-          <t>Operations (Shopfloor): Freigabe Leitung Produktion, P76-Import T76K912718</t>
+          <t>Operations (Shopfloor): SAP-Abgleich läuft seit 09.10.; Abteilungen für 1'912 Aufträge klären, Freigabe Leitung Produktion</t>
         </is>
       </c>
       <c r="C54" s="19" t="inlineStr">
@@ -1375,12 +1375,12 @@
       </c>
       <c r="D54" s="16" t="inlineStr">
         <is>
-          <t>Ingo / Leitung Produktion</t>
+          <t>Leitung Produktion</t>
         </is>
       </c>
       <c r="E54" s="18" t="inlineStr">
         <is>
-          <t>07.10.2026</t>
+          <t>09.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SAP T76: ZM_OFFENE_KDAUF comparison with variants and background mode, docs (notes, learnings, router, baum, Wochen_Todo, coordination)
CMP reads variants with MOVE_OR_WRITE = 'M', can schedule itself as background job (P_BG)
and show the stored result (P_ZEIG), because BI UPDATE hits the 600 s dialog limit. OPT counts
flow calls without invoice rows. Learnings: original not reproducible against itself,
repeated object catalog trap, variant display format, dialog TIME_OUT, substring dump.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -594,7 +594,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Stand 09.10.2026  ·  Ingo Kohler</t>
+          <t>Stand 12.10.2026  ·  Ingo Kohler</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 64 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 19 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 20.</t>
+          <t>Hinter dieser Seite stehen 65 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 19 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 20.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wochen_Todo: close rows 10, 12, 90 with evidence, annotate 26, 55, 82
10: Ann-Katrin confirmed the Exklusiv meaning on 08.10. 14:40.
12: superseded by row 56 (acceptance runs as test meeting, invite 12.10.).
90: ZC23 performance done with row 93 (ZM_OFFENE_KDAUF, 173 s -> 4.5 s).
26/55/82: mail/Teams findings added, rows stay open.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -594,7 +594,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Stand 12.10.2026  ·  Ingo Kohler</t>
+          <t>Stand 13.10.2026  ·  Ingo Kohler</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 65 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 19 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 20.</t>
+          <t>Hinter dieser Seite stehen 62 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 19 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 22.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs: Shopfloor field mapping from Excel 2026-10-14 (b613f7c), section 12, Wochen_Todo 87, deploy pending
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -594,7 +594,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Stand 13.10.2026  ·  Ingo Kohler</t>
+          <t>Stand 14.10.2026  ·  Ingo Kohler</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 63 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 19 auf andere, 13 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 23.</t>
+          <t>Hinter dieser Seite stehen 63 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 19 auf andere, 13 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 15.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wochen_Todo review 2026-10-15: rows 36, 87, 95, 96 updated; new 98 (check Einkauf delta 14.10), 99 (collaboration Fabio), 100 (password hashes out of repo), 101 (start page/header, done)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -594,7 +594,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Stand 14.10.2026  ·  Ingo Kohler</t>
+          <t>Stand 15.10.2026  ·  Ingo Kohler</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 65 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 19 auf andere, 13 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 15.</t>
+          <t>Hinter dieser Seite stehen 68 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 20 auf andere, 13 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 13.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs: Shopfloor package 2026-10-16 in repo (section 14), baum, lastchange, Wochen_Todo 107, learning; deploy waits for VPN
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -594,7 +594,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Stand 15.10.2026  ·  Ingo Kohler</t>
+          <t>Stand 16.10.2026  ·  Ingo Kohler</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 72 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 22 auf andere, 13 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 14.</t>
+          <t>Hinter dieser Seite stehen 73 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 22 auf andere, 13 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 7.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs: Shopfloor quantities on production day, DW prod, rebooking 15.-19.10., deploy 10:04, learnings (weekend zeros, X-User header, wrong SAP session); ZLO03 T76 copy report
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -594,7 +594,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Stand 16.10.2026  ·  Ingo Kohler</t>
+          <t>Stand 19.10.2026  ·  Ingo Kohler</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 72 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 22 auf andere, 13 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 10.</t>
+          <t>Hinter dieser Seite stehen 73 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 22 auf andere, 13 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 10.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Project status 2026-10-19: Wochen_Todo (ZLO03 waits for import, ZC23 and Fiori done in P76, Shopfloor package done, new rows Erfasst/DCP/time entry), Status_kurz, PROJEKTSTATUS PM-01
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -569,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -603,10 +603,10 @@
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="B4" s="4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D4" s="6" t="n">
         <v>12</v>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 73 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 22 auf andere, 13 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 10.</t>
+          <t>Hinter dieser Seite stehen 73 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 21 auf andere, 13 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 13.</t>
         </is>
       </c>
     </row>
@@ -1132,390 +1132,448 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="22" customHeight="1">
-      <c r="B39" s="14" t="inlineStr">
+    <row r="38" ht="20" customHeight="1">
+      <c r="B38" s="16" t="inlineStr">
+        <is>
+          <t>Stücklisten-Netz „Gehirn“ im Spend-Aufriss (Prototyp)</t>
+        </is>
+      </c>
+      <c r="C38" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D38" s="16" t="inlineStr"/>
+      <c r="E38" s="18" t="inlineStr">
+        <is>
+          <t>16.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="B40" s="14" t="inlineStr">
         <is>
           <t>SAP</t>
         </is>
       </c>
-      <c r="C39" s="15" t="n"/>
-      <c r="D39" s="15" t="n"/>
-      <c r="E39" s="15" t="n"/>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="B40" s="16" t="inlineStr">
-        <is>
-          <t>ZZPRDAT Produktionsdatum: gemeinsamer Test</t>
-        </is>
-      </c>
-      <c r="C40" s="20" t="inlineStr">
-        <is>
-          <t>Läuft</t>
-        </is>
-      </c>
-      <c r="D40" s="16" t="inlineStr">
-        <is>
-          <t>Test 12.10. (Lucas, Marco, Adil)</t>
-        </is>
-      </c>
-      <c r="E40" s="18" t="inlineStr">
-        <is>
-          <t>01.10.2026</t>
-        </is>
-      </c>
+      <c r="C40" s="15" t="n"/>
+      <c r="D40" s="15" t="n"/>
+      <c r="E40" s="15" t="n"/>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="B41" s="16" t="inlineStr">
         <is>
-          <t>ZLO03 Mengen und Materialien: Test und Transport</t>
-        </is>
-      </c>
-      <c r="C41" s="22" t="inlineStr">
-        <is>
-          <t>Offen</t>
+          <t>ZZPRDAT Produktionsdatum: gemeinsamer Test</t>
+        </is>
+      </c>
+      <c r="C41" s="20" t="inlineStr">
+        <is>
+          <t>Läuft</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>Ingo</t>
+          <t>Test verschoben auf Woche 26.10. (Lucas, Marco, Adil)</t>
         </is>
       </c>
       <c r="E41" s="18" t="inlineStr">
         <is>
-          <t>14.08.2026</t>
+          <t>12.10.2026</t>
         </is>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>ZC12 Nullmengen: Fehlersuche einschalten</t>
-        </is>
-      </c>
-      <c r="C42" s="22" t="inlineStr">
-        <is>
-          <t>Offen</t>
+          <t>ZLO03: Fehler „offene MK 0 / Komponente fehlt“ behoben, in T76 am nachgestellten Fall bestätigt</t>
+        </is>
+      </c>
+      <c r="C42" s="19" t="inlineStr">
+        <is>
+          <t>Wartet</t>
         </is>
       </c>
       <c r="D42" s="16" t="inlineStr">
         <is>
-          <t>Ingo</t>
+          <t>Import T76K912742 nach P76 (Ingo)</t>
         </is>
       </c>
       <c r="E42" s="18" t="inlineStr">
         <is>
-          <t>07.09.2026</t>
+          <t>19.10.2026</t>
         </is>
       </c>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="B43" s="16" t="inlineStr">
         <is>
+          <t>ZC12 Nullmengen: Fehlersuche einschalten</t>
+        </is>
+      </c>
+      <c r="C43" s="22" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="D43" s="16" t="inlineStr">
+        <is>
+          <t>Ingo</t>
+        </is>
+      </c>
+      <c r="E43" s="18" t="inlineStr">
+        <is>
+          <t>07.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="B44" s="16" t="inlineStr">
+        <is>
           <t>ZRL2 Mengenrabatt Trafag AT</t>
         </is>
       </c>
-      <c r="C43" s="17" t="inlineStr">
+      <c r="C44" s="17" t="inlineStr">
         <is>
           <t>Bereit</t>
         </is>
       </c>
-      <c r="D43" s="16" t="inlineStr"/>
-      <c r="E43" s="18" t="inlineStr">
+      <c r="D44" s="16" t="inlineStr"/>
+      <c r="E44" s="18" t="inlineStr">
         <is>
           <t>30.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="22" customHeight="1">
-      <c r="B45" s="14" t="inlineStr">
+    <row r="45" ht="20" customHeight="1">
+      <c r="B45" s="16" t="inlineStr">
+        <is>
+          <t>ZC23: Materialanteil und Arbeit CZ, 3,5-mal schneller gerechnet, Fiori-App-Anschluss</t>
+        </is>
+      </c>
+      <c r="C45" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D45" s="16" t="inlineStr"/>
+      <c r="E45" s="18" t="inlineStr">
+        <is>
+          <t>16.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="B47" s="14" t="inlineStr">
         <is>
           <t>Railway</t>
         </is>
       </c>
-      <c r="C45" s="15" t="n"/>
-      <c r="D45" s="15" t="n"/>
-      <c r="E45" s="15" t="n"/>
-    </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="B46" s="16" t="inlineStr">
+      <c r="C47" s="15" t="n"/>
+      <c r="D47" s="15" t="n"/>
+      <c r="E47" s="15" t="n"/>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="B48" s="16" t="inlineStr">
         <is>
           <t>Umsatz-Gesamtsicht aller Standorte</t>
         </is>
       </c>
-      <c r="C46" s="17" t="inlineStr">
+      <c r="C48" s="17" t="inlineStr">
         <is>
           <t>Bereit</t>
         </is>
       </c>
-      <c r="D46" s="16" t="inlineStr"/>
-      <c r="E46" s="18" t="inlineStr">
+      <c r="D48" s="16" t="inlineStr"/>
+      <c r="E48" s="18" t="inlineStr">
         <is>
           <t>29.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="B47" s="16" t="inlineStr">
+    <row r="49" ht="20" customHeight="1">
+      <c r="B49" s="16" t="inlineStr">
         <is>
           <t>Top-15-Kunden und Schweiz bestätigen</t>
         </is>
       </c>
-      <c r="C47" s="19" t="inlineStr">
+      <c r="C49" s="19" t="inlineStr">
         <is>
           <t>Wartet</t>
         </is>
       </c>
-      <c r="D47" s="16" t="inlineStr">
+      <c r="D49" s="16" t="inlineStr">
         <is>
           <t>Andreas / Patrik</t>
         </is>
       </c>
-      <c r="E47" s="18" t="inlineStr">
+      <c r="E49" s="18" t="inlineStr">
         <is>
           <t>29.09.2026</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="22" customHeight="1">
-      <c r="B49" s="14" t="inlineStr">
+    <row r="51" ht="22" customHeight="1">
+      <c r="B51" s="14" t="inlineStr">
         <is>
           <t>Plattform</t>
         </is>
       </c>
-      <c r="C49" s="15" t="n"/>
-      <c r="D49" s="15" t="n"/>
-      <c r="E49" s="15" t="n"/>
-    </row>
-    <row r="50" ht="20" customHeight="1">
-      <c r="B50" s="16" t="inlineStr">
-        <is>
-          <t>Webapp schneller</t>
-        </is>
-      </c>
-      <c r="C50" s="17" t="inlineStr">
-        <is>
-          <t>Bereit</t>
-        </is>
-      </c>
-      <c r="D50" s="16" t="inlineStr"/>
-      <c r="E50" s="18" t="inlineStr">
-        <is>
-          <t>28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="20" customHeight="1">
-      <c r="B51" s="16" t="inlineStr">
-        <is>
-          <t>Netzwerk-Reiter: Netzkarte, Verfügbarkeit, Netz oder Daten, Sicherheit</t>
-        </is>
-      </c>
-      <c r="C51" s="17" t="inlineStr">
-        <is>
-          <t>Bereit</t>
-        </is>
-      </c>
-      <c r="D51" s="16" t="inlineStr"/>
-      <c r="E51" s="18" t="inlineStr">
-        <is>
-          <t>02.10.2026</t>
-        </is>
-      </c>
+      <c r="C51" s="15" t="n"/>
+      <c r="D51" s="15" t="n"/>
+      <c r="E51" s="15" t="n"/>
     </row>
     <row r="52" ht="20" customHeight="1">
       <c r="B52" s="16" t="inlineStr">
         <is>
-          <t>AD-Computerkonten im Netzwerk-Reiter einschalten</t>
-        </is>
-      </c>
-      <c r="C52" s="21" t="inlineStr">
-        <is>
-          <t>Erledigt</t>
+          <t>Webapp schneller</t>
+        </is>
+      </c>
+      <c r="C52" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
         </is>
       </c>
       <c r="D52" s="16" t="inlineStr"/>
       <c r="E52" s="18" t="inlineStr">
         <is>
-          <t>02.10.2026</t>
+          <t>28.09.2026</t>
         </is>
       </c>
     </row>
     <row r="53" ht="20" customHeight="1">
       <c r="B53" s="16" t="inlineStr">
         <is>
-          <t>Server im Dauerbetrieb</t>
-        </is>
-      </c>
-      <c r="C53" s="19" t="inlineStr">
-        <is>
-          <t>Wartet</t>
-        </is>
-      </c>
-      <c r="D53" s="16" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
+          <t>Netzwerk-Reiter: Netzkarte, Verfügbarkeit, Netz oder Daten, Sicherheit</t>
+        </is>
+      </c>
+      <c r="C53" s="17" t="inlineStr">
+        <is>
+          <t>Bereit</t>
+        </is>
+      </c>
+      <c r="D53" s="16" t="inlineStr"/>
       <c r="E53" s="18" t="inlineStr">
         <is>
-          <t>28.09.2026</t>
+          <t>02.10.2026</t>
         </is>
       </c>
     </row>
     <row r="54" ht="20" customHeight="1">
       <c r="B54" s="16" t="inlineStr">
         <is>
-          <t>Operations (Shopfloor): SAP-Abgleich läuft seit 09.10.; Abteilungen für 1'912 Aufträge klären, Freigabe Leitung Produktion</t>
-        </is>
-      </c>
-      <c r="C54" s="19" t="inlineStr">
-        <is>
-          <t>Wartet</t>
-        </is>
-      </c>
-      <c r="D54" s="16" t="inlineStr">
-        <is>
-          <t>Leitung Produktion</t>
-        </is>
-      </c>
+          <t>AD-Computerkonten im Netzwerk-Reiter einschalten</t>
+        </is>
+      </c>
+      <c r="C54" s="21" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D54" s="16" t="inlineStr"/>
       <c r="E54" s="18" t="inlineStr">
         <is>
-          <t>09.10.2026</t>
+          <t>02.10.2026</t>
         </is>
       </c>
     </row>
     <row r="55" ht="20" customHeight="1">
       <c r="B55" s="16" t="inlineStr">
         <is>
-          <t>Trafag Reddit: Forum mit Abstimmung, für alle sichtbar</t>
-        </is>
-      </c>
-      <c r="C55" s="20" t="inlineStr">
-        <is>
-          <t>Läuft</t>
+          <t>Server im Dauerbetrieb</t>
+        </is>
+      </c>
+      <c r="C55" s="19" t="inlineStr">
+        <is>
+          <t>Wartet</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>Ingo: Ankündigung entscheiden</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="E55" s="18" t="inlineStr">
         <is>
-          <t>09.10.2026</t>
+          <t>28.09.2026</t>
         </is>
       </c>
     </row>
     <row r="56" ht="20" customHeight="1">
       <c r="B56" s="16" t="inlineStr">
         <is>
+          <t>Operations (Shopfloor): für alle offen, Mengen aus SAP auf dem Produktionstag (Logistik, SEH, TR5, DW), ZD05 04:00/12:45</t>
+        </is>
+      </c>
+      <c r="C56" s="20" t="inlineStr">
+        <is>
+          <t>Läuft</t>
+        </is>
+      </c>
+      <c r="D56" s="16" t="inlineStr">
+        <is>
+          <t>Fabio: TX-Arbeitsplatz; Ingo: TX-Vorrat aus ZC22 bauen</t>
+        </is>
+      </c>
+      <c r="E56" s="18" t="inlineStr">
+        <is>
+          <t>19.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="B57" s="16" t="inlineStr">
+        <is>
+          <t>Trafag Reddit: Forum mit Abstimmung, für alle sichtbar</t>
+        </is>
+      </c>
+      <c r="C57" s="20" t="inlineStr">
+        <is>
+          <t>Läuft</t>
+        </is>
+      </c>
+      <c r="D57" s="16" t="inlineStr">
+        <is>
+          <t>Ingo: Ankündigung entscheiden</t>
+        </is>
+      </c>
+      <c r="E57" s="18" t="inlineStr">
+        <is>
+          <t>09.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="B58" s="16" t="inlineStr">
+        <is>
           <t>Trafag Projekte: Board, Backlog/Sprints, Zeitachse, Kalender, Diagramme</t>
         </is>
       </c>
-      <c r="C56" s="20" t="inlineStr">
+      <c r="C58" s="20" t="inlineStr">
         <is>
           <t>Läuft</t>
         </is>
       </c>
-      <c r="D56" s="16" t="inlineStr">
+      <c r="D58" s="16" t="inlineStr">
         <is>
           <t>Ingo: erstes echtes Projekt anlegen</t>
         </is>
       </c>
-      <c r="E56" s="18" t="inlineStr">
+      <c r="E58" s="18" t="inlineStr">
         <is>
           <t>09.10.2026</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="22" customHeight="1">
-      <c r="B58" s="14" t="inlineStr">
+    <row r="60" ht="22" customHeight="1">
+      <c r="B60" s="14" t="inlineStr">
         <is>
           <t>Projekte</t>
         </is>
       </c>
-      <c r="C58" s="15" t="n"/>
-      <c r="D58" s="15" t="n"/>
-      <c r="E58" s="15" t="n"/>
-    </row>
-    <row r="59" ht="20" customHeight="1">
-      <c r="B59" s="16" t="inlineStr">
+      <c r="C60" s="15" t="n"/>
+      <c r="D60" s="15" t="n"/>
+      <c r="E60" s="15" t="n"/>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="B61" s="16" t="inlineStr">
         <is>
           <t>Smartsheet-Ablösung, Power-BI-Verantwortliche, Data Lake</t>
         </is>
       </c>
-      <c r="C59" s="22" t="inlineStr">
+      <c r="C61" s="22" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="D59" s="16" t="inlineStr">
+      <c r="D61" s="16" t="inlineStr">
         <is>
           <t>noch nicht gestartet</t>
         </is>
       </c>
-      <c r="E59" s="18" t="inlineStr">
+      <c r="E61" s="18" t="inlineStr">
         <is>
           <t>29.09.2026</t>
         </is>
       </c>
-    </row>
-    <row r="61" ht="22" customHeight="1">
-      <c r="B61" s="14" t="inlineStr">
-        <is>
-          <t>Logistik</t>
-        </is>
-      </c>
-      <c r="C61" s="15" t="n"/>
-      <c r="D61" s="15" t="n"/>
-      <c r="E61" s="15" t="n"/>
     </row>
     <row r="62" ht="20" customHeight="1">
       <c r="B62" s="16" t="inlineStr">
         <is>
+          <t>DCP: Testphase freigegeben, nächste Schritte</t>
+        </is>
+      </c>
+      <c r="C62" s="22" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="D62" s="16" t="inlineStr">
+        <is>
+          <t>Klären, worum es geht (Ingo)</t>
+        </is>
+      </c>
+      <c r="E62" s="18" t="inlineStr">
+        <is>
+          <t>19.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="22" customHeight="1">
+      <c r="B64" s="14" t="inlineStr">
+        <is>
+          <t>Logistik</t>
+        </is>
+      </c>
+      <c r="C64" s="15" t="n"/>
+      <c r="D64" s="15" t="n"/>
+      <c r="E64" s="15" t="n"/>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="B65" s="16" t="inlineStr">
+        <is>
           <t>ABAP-Transport Prüfbefund Logistik live (Warenausgangszeit, Kapazität)</t>
         </is>
       </c>
-      <c r="C62" s="19" t="inlineStr">
+      <c r="C65" s="19" t="inlineStr">
         <is>
           <t>Wartet</t>
         </is>
       </c>
-      <c r="D62" s="16" t="inlineStr">
+      <c r="D65" s="16" t="inlineStr">
         <is>
           <t>SE11-Prüfung KBED, T76-Transport</t>
         </is>
       </c>
-      <c r="E62" s="18" t="inlineStr">
+      <c r="E65" s="18" t="inlineStr">
         <is>
           <t>05.10.2026</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="20" customHeight="1">
-      <c r="B63" s="16" t="inlineStr">
+    <row r="66" ht="20" customHeight="1">
+      <c r="B66" s="16" t="inlineStr">
         <is>
           <t>ZM_OFFENE_FAUF mit Bedarfsverursacher (T76K912714 am 09.10. in P76)</t>
         </is>
       </c>
-      <c r="C63" s="20" t="inlineStr">
+      <c r="C66" s="20" t="inlineStr">
         <is>
           <t>Läuft</t>
         </is>
       </c>
-      <c r="D63" s="16" t="inlineStr">
+      <c r="D66" s="16" t="inlineStr">
         <is>
           <t>Fabio: Layout in P76 prüfen, Fall BANF Werk 1200</t>
         </is>
       </c>
-      <c r="E63" s="18" t="inlineStr">
+      <c r="E66" s="18" t="inlineStr">
         <is>
           <t>09.10.2026</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="26" customHeight="1">
-      <c r="B65" s="23" t="inlineStr">
+    <row r="68" ht="26" customHeight="1">
+      <c r="B68" s="23" t="inlineStr">
         <is>
           <t>Bereit = erledigt und in Betrieb · Läuft = in Arbeit · Wartet = braucht eine andere Person · Offen = noch nicht begonnen oder Entscheid von Ingo. Details und Nachweise: Wochen_Todo.xlsx.</t>
         </is>
@@ -1524,7 +1582,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B65:E65"/>
+    <mergeCell ref="B68:E68"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Docs: Word summary GIB Dispo-Cockpit module DCP (what it does, rollout P76, overlap with cockpit); Wochen_Todo 112 and Status_kurz updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -606,13 +606,13 @@
         <v>16</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D4" s="6" t="n">
         <v>12</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -1499,17 +1499,17 @@
     <row r="62" ht="20" customHeight="1">
       <c r="B62" s="16" t="inlineStr">
         <is>
-          <t>DCP: Testphase freigegeben, nächste Schritte</t>
-        </is>
-      </c>
-      <c r="C62" s="22" t="inlineStr">
-        <is>
-          <t>Offen</t>
+          <t>GIB Dispo-Cockpit DCP (SAP-Add-on Planung): Rollout P76 in 1,5 bis 2 Wochen</t>
+        </is>
+      </c>
+      <c r="C62" s="20" t="inlineStr">
+        <is>
+          <t>Läuft</t>
         </is>
       </c>
       <c r="D62" s="16" t="inlineStr">
         <is>
-          <t>Klären, worum es geht (Ingo)</t>
+          <t>Projekt (Sergio, Oscar Schwark): Umfang, Rollen</t>
         </is>
       </c>
       <c r="E62" s="18" t="inlineStr">

</xml_diff>

<commit_message>
SAP T76/200: test user UBIG with GIB role /GIB/DCP_SUPERVISOR only; GIB roles and transactions documented, SapProbe pitfall in learnings; Wochen_Todo 112 and Status_kurz (modules installed, pilot done)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -1499,7 +1499,7 @@
     <row r="62" ht="20" customHeight="1">
       <c r="B62" s="16" t="inlineStr">
         <is>
-          <t>GIB Dispo-Cockpit DCP (SAP-Add-on Planung): Rollout P76 in 1,5 bis 2 Wochen</t>
+          <t>GIB Dispo-Cockpit DCP (SAP-Add-on Planung): Module installiert, Pilot abgeschlossen, Testuser UBIG in T76/200</t>
         </is>
       </c>
       <c r="C62" s="20" t="inlineStr">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="D62" s="16" t="inlineStr">
         <is>
-          <t>Projekt (Sergio, Oscar Schwark): Umfang, Rollen</t>
+          <t>Ingo: Kennwort UBIG setzen und testen; Projekt: Umfang, Rollen</t>
         </is>
       </c>
       <c r="E62" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Wochen_Todo 113 done: time entry 15.10. added by Ingo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -594,7 +594,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Stand 19.10.2026  ·  Ingo Kohler</t>
+          <t>Stand 20.10.2026  ·  Ingo Kohler</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 73 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 21 auf andere, 13 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 13.</t>
+          <t>Hinter dieser Seite stehen 72 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 21 auf andere, 13 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 14.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ZLO03 FIX 19: columns REACH, SVHC, PFAS content from class Z_PACK_REGULATION (request Florian), active in T76 in transport T76K912742 together with FIX 12; per-field findings T76/P76 (no RoHS in P76), P76 read scripts, Wochen_Todo 9/114, Status_kurz, PM-01
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 72 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 21 auf andere, 13 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 14.</t>
+          <t>Hinter dieser Seite stehen 73 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 21 auf andere, 13 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 14.</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1185,7 @@
     <row r="42" ht="20" customHeight="1">
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>ZLO03: Fehler „offene MK 0 / Komponente fehlt“ behoben, in T76 am nachgestellten Fall bestätigt</t>
+          <t>ZLO03: Fehler „offene MK 0“ behoben (FIX 12) und Spalten REACH/SVHC/PFAS neu (FIX 19), beide in T76K912742</t>
         </is>
       </c>
       <c r="C42" s="19" t="inlineStr">
@@ -1195,12 +1195,12 @@
       </c>
       <c r="D42" s="16" t="inlineStr">
         <is>
-          <t>Import T76K912742 nach P76 (Ingo)</t>
+          <t>Import nach P76 (Ingo); RoHS-Merkmal (Adil)</t>
         </is>
       </c>
       <c r="E42" s="18" t="inlineStr">
         <is>
-          <t>19.10.2026</t>
+          <t>20.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs: SAP PS introduction and demo in T76 (project DEMO-PS, time on WBS via KB21N, CJI3), findings (PS not set up for Trafag), transactions, verdict; 14 screenshots; learnings (HardCopy minimized window, client of task, empty cscript args, KB21N subscreen, local customizing request)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -569,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E68"/>
+  <dimension ref="A1:E69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -606,7 +606,7 @@
         <v>16</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D4" s="6" t="n">
         <v>12</v>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 73 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 21 auf andere, 13 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 14.</t>
+          <t>Hinter dieser Seite stehen 74 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 21 auf andere, 13 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 14.</t>
         </is>
       </c>
     </row>
@@ -1518,62 +1518,84 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="22" customHeight="1">
-      <c r="B64" s="14" t="inlineStr">
+    <row r="63" ht="20" customHeight="1">
+      <c r="B63" s="16" t="inlineStr">
+        <is>
+          <t>SAP PS: Demo in T76, Fazit einfach zu bedienen, Einfuehrung mittel (PS nicht eingerichtet, Zeit heute in rexx)</t>
+        </is>
+      </c>
+      <c r="C63" s="20" t="inlineStr">
+        <is>
+          <t>Läuft</t>
+        </is>
+      </c>
+      <c r="D63" s="16" t="inlineStr">
+        <is>
+          <t>Ingo: Folien, P76-Pruefung; Philip Steiger</t>
+        </is>
+      </c>
+      <c r="E63" s="18" t="inlineStr">
+        <is>
+          <t>20.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="22" customHeight="1">
+      <c r="B65" s="14" t="inlineStr">
         <is>
           <t>Logistik</t>
         </is>
       </c>
-      <c r="C64" s="15" t="n"/>
-      <c r="D64" s="15" t="n"/>
-      <c r="E64" s="15" t="n"/>
-    </row>
-    <row r="65" ht="20" customHeight="1">
-      <c r="B65" s="16" t="inlineStr">
-        <is>
-          <t>ABAP-Transport Prüfbefund Logistik live (Warenausgangszeit, Kapazität)</t>
-        </is>
-      </c>
-      <c r="C65" s="19" t="inlineStr">
-        <is>
-          <t>Wartet</t>
-        </is>
-      </c>
-      <c r="D65" s="16" t="inlineStr">
-        <is>
-          <t>SE11-Prüfung KBED, T76-Transport</t>
-        </is>
-      </c>
-      <c r="E65" s="18" t="inlineStr">
-        <is>
-          <t>05.10.2026</t>
-        </is>
-      </c>
+      <c r="C65" s="15" t="n"/>
+      <c r="D65" s="15" t="n"/>
+      <c r="E65" s="15" t="n"/>
     </row>
     <row r="66" ht="20" customHeight="1">
       <c r="B66" s="16" t="inlineStr">
         <is>
+          <t>ABAP-Transport Prüfbefund Logistik live (Warenausgangszeit, Kapazität)</t>
+        </is>
+      </c>
+      <c r="C66" s="19" t="inlineStr">
+        <is>
+          <t>Wartet</t>
+        </is>
+      </c>
+      <c r="D66" s="16" t="inlineStr">
+        <is>
+          <t>SE11-Prüfung KBED, T76-Transport</t>
+        </is>
+      </c>
+      <c r="E66" s="18" t="inlineStr">
+        <is>
+          <t>05.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="20" customHeight="1">
+      <c r="B67" s="16" t="inlineStr">
+        <is>
           <t>ZM_OFFENE_FAUF mit Bedarfsverursacher (T76K912714 am 09.10. in P76)</t>
         </is>
       </c>
-      <c r="C66" s="20" t="inlineStr">
+      <c r="C67" s="20" t="inlineStr">
         <is>
           <t>Läuft</t>
         </is>
       </c>
-      <c r="D66" s="16" t="inlineStr">
+      <c r="D67" s="16" t="inlineStr">
         <is>
           <t>Fabio: Layout in P76 prüfen, Fall BANF Werk 1200</t>
         </is>
       </c>
-      <c r="E66" s="18" t="inlineStr">
+      <c r="E67" s="18" t="inlineStr">
         <is>
           <t>09.10.2026</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="26" customHeight="1">
-      <c r="B68" s="23" t="inlineStr">
+    <row r="69" ht="26" customHeight="1">
+      <c r="B69" s="23" t="inlineStr">
         <is>
           <t>Bereit = erledigt und in Betrieb · Läuft = in Arbeit · Wartet = braucht eine andere Person · Offen = noch nicht begonnen oder Entscheid von Ingo. Details und Nachweise: Wochen_Todo.xlsx.</t>
         </is>
@@ -1582,7 +1604,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B68:E68"/>
+    <mergeCell ref="B69:E69"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Status: closing round dashboard and data lake invited (20.10.), Wochen_Todo 116
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -606,13 +606,13 @@
         <v>16</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D4" s="6" t="n">
         <v>12</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 74 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 21 auf andere, 13 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 14.</t>
+          <t>Hinter dieser Seite stehen 75 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 21 auf andere, 13 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 14.</t>
         </is>
       </c>
     </row>
@@ -1477,22 +1477,22 @@
     <row r="61" ht="20" customHeight="1">
       <c r="B61" s="16" t="inlineStr">
         <is>
-          <t>Smartsheet-Ablösung, Power-BI-Verantwortliche, Data Lake</t>
-        </is>
-      </c>
-      <c r="C61" s="22" t="inlineStr">
-        <is>
-          <t>Offen</t>
+          <t>Abschlussrunde Dashboard und Data Lake (Finance, Einkauf, Supply Chain, HR, Sales, 90 Min.); Smartsheet-Ablösung, Power-BI-Verantwortliche</t>
+        </is>
+      </c>
+      <c r="C61" s="20" t="inlineStr">
+        <is>
+          <t>Läuft</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
         <is>
-          <t>noch nicht gestartet</t>
+          <t>Einladung am 20.10. verschickt (Ingo)</t>
         </is>
       </c>
       <c r="E61" s="18" t="inlineStr">
         <is>
-          <t>29.09.2026</t>
+          <t>20.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Status: Wochen_Todo 117 (uncommitted Finance_All automation, decision Ingo), 118 (Qdrant reindex script robustness), note row 15; code vs docs check since 01.10. (no app code after deploy c3c45cd); Qdrant index rebuilt (4245 sections); learnings
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -594,7 +594,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Stand 20.10.2026  ·  Ingo Kohler</t>
+          <t>Stand 21.10.2026  ·  Ingo Kohler</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 75 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 21 auf andere, 13 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 14.</t>
+          <t>Hinter dieser Seite stehen 77 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 23 auf andere, 13 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 13.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ZLO03 FIX 20: "broken Excel" is Excel blocking tab text saved as .xls (group policy ExtensionHardening = 2); download_dialog now saves .txt and opens it with excel.exe (fallback default program); T76 active, read back identical, run opens Excel, content unchanged; transport T76K912742; docs, Wochen_Todo 114/119
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -594,7 +594,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Stand 21.10.2026  ·  Ingo Kohler</t>
+          <t>Stand 22.10.2026  ·  Ingo Kohler</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 77 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 23 auf andere, 13 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 13.</t>
+          <t>Hinter dieser Seite stehen 78 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 23 auf andere, 13 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 13.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Einkauf product group like ZM_OFFENE_KDAUF: own MRP controller MARC-DISPO (plant 1100) -> ZDISPO_GRP/ZDISPO_SPART -> exactly one group per material, no inheritance via where-used and no 1/n split (decision Ingo 2026-10-26); ambiguous SAP rules take the lowest group code; new column MarcDispo filled by full load and delta; tests; docs
Mein Gebieter, die Produktgruppe kommt jetzt wie im Report aus dem eigenen Disponenten.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -594,7 +594,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Stand 22.10.2026  ·  Ingo Kohler</t>
+          <t>Stand 26.10.2026  ·  Ingo Kohler</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 80 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 24 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 14.</t>
+          <t>Hinter dieser Seite stehen 80 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 24 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 13.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs: ZZPRDAT Live-Pruefung T76 vom 26.10. nachgefuehrt, mein Gebieter
Quelltext in T76 identisch mit saptasks/zzprdat/produktiv, letzte Aenderung 07.09.,
BAdI aktiv, T76K912490/491 offen. Sieben Testauftraege TAN/FPA (1241831 bis 1241844)
im Transportplan dokumentiert. PM-03, Status_kurz, Wochen_Todo 56 samt xlsx, rag,
lastchange, zwei LEARNINGS-Zeilen. SAP nur lesend, kein Deploy.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -594,7 +594,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Stand 26.10.2026  ·  Ingo Kohler</t>
+          <t>Stand 27.10.2026  ·  Ingo Kohler</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 80 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 24 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 13.</t>
+          <t>Hinter dieser Seite stehen 80 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 24 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 11.</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>Test verschoben auf Woche 26.10. (Lucas, Marco, Adil)</t>
+          <t>Abnahmetest Woche ab 26.10. (Lucas, Marco, Adil); Technik am 26.10. live bestätigt, unverändert seit 07.09.</t>
         </is>
       </c>
       <c r="E41" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Docs: Kostenstruktur Material je Produktgruppe (Sitzung 28.10.), Phase 1 8653f6b, Phase 2 offen, Wochen_Todo 123, mein Gebieter
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -594,7 +594,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Stand 27.10.2026  ·  Ingo Kohler</t>
+          <t>Stand 28.10.2026  ·  Ingo Kohler</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 80 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 24 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 11.</t>
+          <t>Hinter dieser Seite stehen 81 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 24 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 10.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs: Widersprueche in allen Markdown-Dateien aufgeloest (Router, RAG, Fachdateien, saptasks, Handbuch, PROJEKTSTATUS), Issue-Log ISS-004/006.1/007.2, Wochen_Todo/Status_kurz nachgefuehrt, LEARNINGS, mein Gebieter
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -594,7 +594,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Stand 28.10.2026  ·  Ingo Kohler</t>
+          <t>Stand 29.10.2026  ·  Ingo Kohler</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -612,7 +612,7 @@
         <v>12</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 81 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 24 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 10.</t>
+          <t>Hinter dieser Seite stehen 81 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 25 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 9.</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
     <row r="23" ht="20" customHeight="1">
       <c r="B23" s="16" t="inlineStr">
         <is>
-          <t>Kader 8,1 h, übrige 8,0 h je Arbeitstag</t>
+          <t>Kader (SAP-Mitarbeiterkreis 10) 8,2 h, übrige 8,0 h je Arbeitstag</t>
         </is>
       </c>
       <c r="C23" s="17" t="inlineStr">
@@ -882,7 +882,7 @@
       <c r="D23" s="16" t="inlineStr"/>
       <c r="E23" s="18" t="inlineStr">
         <is>
-          <t>01.10.2026</t>
+          <t>22.10.2026</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1185,7 @@
     <row r="42" ht="20" customHeight="1">
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>ZLO03: Fehler „offene MK 0“ behoben (FIX 12) und Spalten REACH/SVHC/PFAS neu (FIX 19), beide in T76K912742</t>
+          <t>ZLO03: Fehler „offene MK 0“ behoben (FIX 12), Spalten RoHS/REACH/SVHC/PFAS (FIX 19), Download (FIX 20) in T76K912742 (freigegeben 22.10.), .xlsx (FIX 21) in T76K912752</t>
         </is>
       </c>
       <c r="C42" s="19" t="inlineStr">
@@ -1195,12 +1195,12 @@
       </c>
       <c r="D42" s="16" t="inlineStr">
         <is>
-          <t>Import nach P76 (Ingo); RoHS-Merkmal (Adil)</t>
+          <t>Import nach P76 (Ingo); Freigabe T76K912752 (Ingo)</t>
         </is>
       </c>
       <c r="E42" s="18" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>22.10.2026</t>
         </is>
       </c>
     </row>
@@ -1210,19 +1210,19 @@
           <t>ZC12 Nullmengen: Fehlersuche einschalten</t>
         </is>
       </c>
-      <c r="C43" s="22" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="C43" s="21" t="inlineStr">
+        <is>
+          <t>Ruht</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>Ingo</t>
+          <t>Entscheid Ingo 01.10.: nichts tun</t>
         </is>
       </c>
       <c r="E43" s="18" t="inlineStr">
         <is>
-          <t>07.09.2026</t>
+          <t>01.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs: Nachpruefung Finance-Dateien vollstaendig gelesen, Kursumweg A2 (ISS-018) seit Budgetkurs-Standard wirksam, Querbefunde RAG, Status_kurz ZC12, LEARNINGS, Qdrant 4467/4467, mein Gebieter
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -612,7 +612,7 @@
         <v>12</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -1210,14 +1210,14 @@
           <t>ZC12 Nullmengen: Fehlersuche einschalten</t>
         </is>
       </c>
-      <c r="C43" s="21" t="inlineStr">
-        <is>
-          <t>Ruht</t>
+      <c r="C43" s="22" t="inlineStr">
+        <is>
+          <t>Offen</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>Entscheid Ingo 01.10.: nichts tun</t>
+          <t>Ingo (Entscheid 01.10.: Editor in T76 so lassen, nichts tun)</t>
         </is>
       </c>
       <c r="E43" s="18" t="inlineStr">

</xml_diff>

<commit_message>
ZLO03 FIX 22 Top-Down Disponent und Warengruppe (T76K912777), ZC23-Gruppe BM BG_MECHANIK fuer Disponent 026 in P76, Doku, mein Gebieter
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 81 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 25 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 9.</t>
+          <t>Hinter dieser Seite stehen 82 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 26 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 10.</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1185,7 @@
     <row r="42" ht="20" customHeight="1">
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>ZLO03: Fehler „offene MK 0“ behoben (FIX 12), Spalten RoHS/REACH/SVHC/PFAS (FIX 19), Download (FIX 20) in T76K912742 (freigegeben 22.10.), .xlsx (FIX 21) in T76K912752</t>
+          <t>ZLO03: Fehler „offene MK 0“ behoben (FIX 12), Spalten RoHS/REACH/SVHC/PFAS (FIX 19), Download (FIX 20) in T76K912742 (freigegeben 22.10.), .xlsx (FIX 21) in T76K912752 (freigegeben), Disponent/Warengruppe im Top-Down (FIX 22) in T76K912777</t>
         </is>
       </c>
       <c r="C42" s="19" t="inlineStr">
@@ -1195,12 +1195,12 @@
       </c>
       <c r="D42" s="16" t="inlineStr">
         <is>
-          <t>Import nach P76 (Ingo); Freigabe T76K912752 (Ingo)</t>
+          <t>Import nach P76 in dieser Reihenfolge, Freigabe T76K912777 (Ingo)</t>
         </is>
       </c>
       <c r="E42" s="18" t="inlineStr">
         <is>
-          <t>22.10.2026</t>
+          <t>29.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ZLO03 FIX 23 Top-Down Mengen und Stueckkosten in Stuecklisten-Einheit ueber MARM (H05039 KAR/ST, Meldung Armin), T76K912781, Doku, mein Gebieter
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 84 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 26 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 10.</t>
+          <t>Hinter dieser Seite stehen 85 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 27 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 10.</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1185,7 @@
     <row r="42" ht="20" customHeight="1">
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>ZLO03: Fehler „offene MK 0“ behoben (FIX 12), Spalten RoHS/REACH/SVHC/PFAS (FIX 19), Download (FIX 20) in T76K912742 (freigegeben 22.10.), .xlsx (FIX 21) in T76K912752 (freigegeben), Disponent/Warengruppe im Top-Down (FIX 22) in T76K912777</t>
+          <t>ZLO03: Fehler „offene MK 0“ behoben (FIX 12), Spalten RoHS/REACH/SVHC/PFAS (FIX 19), Download (FIX 20) in T76K912742 (freigegeben 22.10.), .xlsx (FIX 21) in T76K912752 (freigegeben), Disponent/Warengruppe im Top-Down (FIX 22) in T76K912777, Stuecklisten-Einheit im Top-Down (FIX 23) in T76K912781</t>
         </is>
       </c>
       <c r="C42" s="19" t="inlineStr">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="D42" s="16" t="inlineStr">
         <is>
-          <t>Import nach P76 in dieser Reihenfolge, Freigabe T76K912777 (Ingo)</t>
+          <t>Import nach P76 in dieser Reihenfolge, Freigabe T76K912781 (Ingo)</t>
         </is>
       </c>
       <c r="E42" s="18" t="inlineStr">

</xml_diff>

<commit_message>
ZLO03 FIX 24: Stueckkosten ungerundet, Textpositionen nicht im Bedarf, Bottom-Up-Details in Stuecklisten-Einheit (T76K912785), fuenf Testlaeufe bestanden, Doku, mein Gebieter
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
+++ b/TrafagSalesExporter/projektmanagement/Status_kurz.xlsx
@@ -594,7 +594,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Stand 29.10.2026  ·  Ingo Kohler</t>
+          <t>Stand 30.10.2026  ·  Ingo Kohler</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -640,7 +640,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Hinter dieser Seite stehen 86 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 27 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 10.</t>
+          <t>Hinter dieser Seite stehen 86 offene Detailpunkte (Wochen_Todo.xlsx). Davon warten 26 auf andere, 14 sind Kleinigkeiten zum Terminieren. In den letzten 14 Tagen erledigt: 9.</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1185,7 @@
     <row r="42" ht="20" customHeight="1">
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>ZLO03: Fehler „offene MK 0“ behoben (FIX 12), Spalten RoHS/REACH/SVHC/PFAS (FIX 19), Download (FIX 20) in T76K912742 (freigegeben 22.10.), .xlsx (FIX 21) in T76K912752 (freigegeben), Disponent/Warengruppe im Top-Down (FIX 22) in T76K912777, Stuecklisten-Einheit im Top-Down (FIX 23) in T76K912781</t>
+          <t>ZLO03: FIX 12 bis 23 (offene MK, RoHS/REACH/SVHC/PFAS, Download .xlsx, Disponent/Warengruppe, Stuecklisten-Einheit) am 29.10. in P76 importiert; FIX 24 (Stueckkosten ungerundet, Textpositionen nicht im Bedarf, Bottom-Up-Details in Stuecklisten-Einheit) in T76K912785, getestet</t>
         </is>
       </c>
       <c r="C42" s="19" t="inlineStr">
@@ -1195,12 +1195,12 @@
       </c>
       <c r="D42" s="16" t="inlineStr">
         <is>
-          <t>Import nach P76 in dieser Reihenfolge, Freigabe T76K912781 (Ingo)</t>
+          <t>Freigabe und Import T76K912785 (Ingo), Armin antworten, Anwender informieren</t>
         </is>
       </c>
       <c r="E42" s="18" t="inlineStr">
         <is>
-          <t>29.10.2026</t>
+          <t>30.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>